<commit_message>
chore: update activity report [2026-04-10 09:44 UTC] via push (run 24236872105)
</commit_message>
<xml_diff>
--- a/github_activity_report.xlsx
+++ b/github_activity_report.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Failure Alerts" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Activity'!$A$1:$Y$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Activity'!$A$1:$Y$28</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Failure Summary'!$A$1:$L$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Failure Alerts'!$A$3:$L$18</definedName>
   </definedNames>
@@ -532,7 +532,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y26"/>
+  <dimension ref="A1:Y28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -540,8 +540,8 @@
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="42" customWidth="1" min="5" max="5"/>
-    <col width="54" customWidth="1" min="6" max="6"/>
-    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="62" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
     <col width="17" customWidth="1" min="9" max="9"/>
     <col width="9" customWidth="1" min="10" max="10"/>
@@ -2418,12 +2418,12 @@
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>4246e5f5bdd0c663224514d45c37457253e6806b</t>
+          <t>aac0b4a033d6b371042ec3f99a213aa53e5d925f</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr">
         <is>
-          <t>test-13</t>
+          <t>test-198</t>
         </is>
       </c>
       <c r="G20" s="6" t="inlineStr">
@@ -2433,7 +2433,7 @@
       </c>
       <c r="H20" s="6" t="inlineStr">
         <is>
-          <t>2026-04-10T09:35:54Z</t>
+          <t>2026-04-10T09:40:50Z</t>
         </is>
       </c>
       <c r="I20" s="6" t="inlineStr">
@@ -2453,7 +2453,7 @@
         </is>
       </c>
       <c r="Q20" s="6" t="n">
-        <v>24236579665</v>
+        <v>24236872105</v>
       </c>
       <c r="R20" s="6" t="inlineStr">
         <is>
@@ -2473,85 +2473,67 @@
       <c r="Y20" s="6" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>git-report</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>vidyakar-whitedev</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>git-report</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>vidyakar-whitedev</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
         <is>
           <t>public</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="D21" s="7" t="inlineStr">
         <is>
           <t>main</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>ff12234265b7ed9747283a1b59735ea5ddda19b5</t>
-        </is>
-      </c>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>test-12</t>
-        </is>
-      </c>
-      <c r="G21" s="2" t="inlineStr">
-        <is>
-          <t>“Vidyakar”</t>
-        </is>
-      </c>
-      <c r="H21" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-10T09:21:24Z</t>
-        </is>
-      </c>
-      <c r="I21" s="2" t="inlineStr">
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>19b0e6e1eadc37093a80d5aa3b43d47cf52cc739</t>
+        </is>
+      </c>
+      <c r="F21" s="7" t="inlineStr">
+        <is>
+          <t>chore: update activity report [2026-04-10 09:36 UTC] via push (run 24236579665)</t>
+        </is>
+      </c>
+      <c r="G21" s="7" t="inlineStr">
+        <is>
+          <t>github-actions[bot]</t>
+        </is>
+      </c>
+      <c r="H21" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-10T09:36:36Z</t>
+        </is>
+      </c>
+      <c r="I21" s="7" t="inlineStr">
         <is>
           <t>main</t>
         </is>
       </c>
-      <c r="J21" s="2" t="inlineStr"/>
-      <c r="K21" s="2" t="inlineStr"/>
-      <c r="L21" s="2" t="inlineStr"/>
-      <c r="M21" s="2" t="inlineStr"/>
-      <c r="N21" s="2" t="inlineStr"/>
-      <c r="O21" s="2" t="inlineStr"/>
-      <c r="P21" s="2" t="inlineStr">
-        <is>
-          <t>GitHub Activity Report</t>
-        </is>
-      </c>
-      <c r="Q21" s="2" t="n">
-        <v>24236015736</v>
-      </c>
-      <c r="R21" s="2" t="inlineStr">
-        <is>
-          <t>push</t>
-        </is>
-      </c>
-      <c r="S21" s="2" t="inlineStr">
-        <is>
-          <t>completed</t>
-        </is>
-      </c>
-      <c r="T21" s="3" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
-      <c r="U21" s="2" t="inlineStr"/>
-      <c r="V21" s="2" t="inlineStr"/>
-      <c r="W21" s="2" t="inlineStr"/>
-      <c r="X21" s="2" t="inlineStr"/>
-      <c r="Y21" s="2" t="inlineStr"/>
+      <c r="J21" s="7" t="inlineStr"/>
+      <c r="K21" s="7" t="inlineStr"/>
+      <c r="L21" s="7" t="inlineStr"/>
+      <c r="M21" s="7" t="inlineStr"/>
+      <c r="N21" s="7" t="inlineStr"/>
+      <c r="O21" s="7" t="inlineStr"/>
+      <c r="P21" s="7" t="inlineStr"/>
+      <c r="Q21" s="7" t="inlineStr"/>
+      <c r="R21" s="7" t="inlineStr"/>
+      <c r="S21" s="7" t="inlineStr"/>
+      <c r="T21" s="7" t="inlineStr"/>
+      <c r="U21" s="7" t="inlineStr"/>
+      <c r="V21" s="7" t="inlineStr"/>
+      <c r="W21" s="7" t="inlineStr"/>
+      <c r="X21" s="7" t="inlineStr"/>
+      <c r="Y21" s="7" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -2576,12 +2558,12 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>75732834dd766afc090c808510eb71c7693015dd</t>
+          <t>4246e5f5bdd0c663224514d45c37457253e6806b</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>test-8</t>
+          <t>test-13</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -2591,7 +2573,7 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>2026-04-10T08:35:13Z</t>
+          <t>2026-04-10T09:35:54Z</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
@@ -2611,7 +2593,7 @@
         </is>
       </c>
       <c r="Q22" s="2" t="n">
-        <v>24234243976</v>
+        <v>24236579665</v>
       </c>
       <c r="R22" s="2" t="inlineStr">
         <is>
@@ -2657,12 +2639,12 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>9d220c5657c48c13ca17102c507b756edbba9215</t>
+          <t>ff12234265b7ed9747283a1b59735ea5ddda19b5</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>test-8</t>
+          <t>test-12</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -2672,7 +2654,7 @@
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>2026-04-10T08:32:22Z</t>
+          <t>2026-04-10T09:21:24Z</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
@@ -2692,7 +2674,7 @@
         </is>
       </c>
       <c r="Q23" s="2" t="n">
-        <v>24234135440</v>
+        <v>24236015736</v>
       </c>
       <c r="R23" s="2" t="inlineStr">
         <is>
@@ -2738,7 +2720,7 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>981fe60621c98393750f79dd815a0ea7e4aed75e</t>
+          <t>75732834dd766afc090c808510eb71c7693015dd</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -2753,7 +2735,7 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>2026-04-10T08:27:06Z</t>
+          <t>2026-04-10T08:35:13Z</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
@@ -2773,7 +2755,7 @@
         </is>
       </c>
       <c r="Q24" s="2" t="n">
-        <v>24233936358</v>
+        <v>24234243976</v>
       </c>
       <c r="R24" s="2" t="inlineStr">
         <is>
@@ -2819,12 +2801,12 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>3cfdf96375ed8ea8c83b95f26b9c87428b8bc8b9</t>
+          <t>9d220c5657c48c13ca17102c507b756edbba9215</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>test-1</t>
+          <t>test-8</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -2834,7 +2816,7 @@
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>2026-04-10T08:18:15Z</t>
+          <t>2026-04-10T08:32:22Z</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
@@ -2854,7 +2836,7 @@
         </is>
       </c>
       <c r="Q25" s="2" t="n">
-        <v>24233616319</v>
+        <v>24234135440</v>
       </c>
       <c r="R25" s="2" t="inlineStr">
         <is>
@@ -2900,12 +2882,12 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>ad211e0513d37204ee54168120dec41978cc6fb4</t>
+          <t>981fe60621c98393750f79dd815a0ea7e4aed75e</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>new code change</t>
+          <t>test-8</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -2915,7 +2897,7 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>2026-04-06T15:32:05Z</t>
+          <t>2026-04-10T08:27:06Z</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
@@ -2935,7 +2917,7 @@
         </is>
       </c>
       <c r="Q26" s="2" t="n">
-        <v>24038137070</v>
+        <v>24233936358</v>
       </c>
       <c r="R26" s="2" t="inlineStr">
         <is>
@@ -2958,8 +2940,170 @@
       <c r="X26" s="2" t="inlineStr"/>
       <c r="Y26" s="2" t="inlineStr"/>
     </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>git-report</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>vidyakar-whitedev</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>3cfdf96375ed8ea8c83b95f26b9c87428b8bc8b9</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>test-1</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>“Vidyakar”</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-10T08:18:15Z</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr"/>
+      <c r="K27" s="2" t="inlineStr"/>
+      <c r="L27" s="2" t="inlineStr"/>
+      <c r="M27" s="2" t="inlineStr"/>
+      <c r="N27" s="2" t="inlineStr"/>
+      <c r="O27" s="2" t="inlineStr"/>
+      <c r="P27" s="2" t="inlineStr">
+        <is>
+          <t>GitHub Activity Report</t>
+        </is>
+      </c>
+      <c r="Q27" s="2" t="n">
+        <v>24233616319</v>
+      </c>
+      <c r="R27" s="2" t="inlineStr">
+        <is>
+          <t>push</t>
+        </is>
+      </c>
+      <c r="S27" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="T27" s="3" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="U27" s="2" t="inlineStr"/>
+      <c r="V27" s="2" t="inlineStr"/>
+      <c r="W27" s="2" t="inlineStr"/>
+      <c r="X27" s="2" t="inlineStr"/>
+      <c r="Y27" s="2" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>git-report</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>vidyakar-whitedev</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>ad211e0513d37204ee54168120dec41978cc6fb4</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>new code change</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>“Vidyakar”</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-06T15:32:05Z</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr"/>
+      <c r="K28" s="2" t="inlineStr"/>
+      <c r="L28" s="2" t="inlineStr"/>
+      <c r="M28" s="2" t="inlineStr"/>
+      <c r="N28" s="2" t="inlineStr"/>
+      <c r="O28" s="2" t="inlineStr"/>
+      <c r="P28" s="2" t="inlineStr">
+        <is>
+          <t>GitHub Activity Report</t>
+        </is>
+      </c>
+      <c r="Q28" s="2" t="n">
+        <v>24038137070</v>
+      </c>
+      <c r="R28" s="2" t="inlineStr">
+        <is>
+          <t>push</t>
+        </is>
+      </c>
+      <c r="S28" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="T28" s="3" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="U28" s="2" t="inlineStr"/>
+      <c r="V28" s="2" t="inlineStr"/>
+      <c r="W28" s="2" t="inlineStr"/>
+      <c r="X28" s="2" t="inlineStr"/>
+      <c r="Y28" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Y26"/>
+  <autoFilter ref="A1:Y28"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4035,7 +4179,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="9" t="inlineStr">
         <is>
-          <t>Generated: 2026-04-10 09:36 UTC</t>
+          <t>Generated: 2026-04-10 09:44 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update activity report [2026-04-11 05:18 UTC] (run 24275511539)
</commit_message>
<xml_diff>
--- a/github_activity_report.xlsx
+++ b/github_activity_report.xlsx
@@ -14,7 +14,7 @@
     <sheet name="Failure Alerts" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Activity'!$A$1:$Z$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Activity'!$A$1:$Z$38</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Failure Summary'!$A$1:$M$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Failure Alerts'!$A$3:$M$19</definedName>
   </definedNames>
@@ -202,13 +202,13 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -618,7 +618,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>2026-04-10 16:37 UTC</t>
+          <t>2026-04-11 05:18 UTC</t>
         </is>
       </c>
     </row>
@@ -630,7 +630,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>2026-03-11 → now</t>
+          <t>2026-03-12 → now</t>
         </is>
       </c>
     </row>
@@ -791,7 +791,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z36"/>
+  <dimension ref="A1:Z38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -977,12 +977,12 @@
       </c>
       <c r="E2" s="15" t="inlineStr">
         <is>
-          <t>93bdf4123cc644f621cecd131589bff39d5376fe</t>
+          <t>c68bea9e4038cecbe103d4f97e57de3e9e0b277f</t>
         </is>
       </c>
       <c r="F2" s="15" t="inlineStr">
         <is>
-          <t>test-249</t>
+          <t>fix: correct typo in demo.txt</t>
         </is>
       </c>
       <c r="G2" s="15" t="inlineStr">
@@ -992,7 +992,7 @@
       </c>
       <c r="H2" s="15" t="inlineStr">
         <is>
-          <t>2026-04-10T16:36:38Z</t>
+          <t>2026-04-11T05:17:03Z</t>
         </is>
       </c>
       <c r="I2" s="15" t="inlineStr">
@@ -1012,7 +1012,7 @@
         </is>
       </c>
       <c r="Q2" s="15" t="n">
-        <v>24253439879</v>
+        <v>24275511539</v>
       </c>
       <c r="R2" s="15" t="inlineStr">
         <is>
@@ -1021,7 +1021,7 @@
       </c>
       <c r="S2" s="15" t="inlineStr">
         <is>
-          <t>2026-04-10T16:36:56Z</t>
+          <t>2026-04-11T05:18:13Z</t>
         </is>
       </c>
       <c r="T2" s="15" t="inlineStr">
@@ -1059,22 +1059,22 @@
       </c>
       <c r="E3" s="16" t="inlineStr">
         <is>
-          <t>b3ea79ed073ed633f20c5321bc134cc65896c901</t>
+          <t>d8fe1f0413e72ae3882ff6057ee827a33bfc8468</t>
         </is>
       </c>
       <c r="F3" s="16" t="inlineStr">
         <is>
-          <t>test-209</t>
+          <t>chore: update activity report [2026-04-10 16:37 UTC] (run 24253439879)</t>
         </is>
       </c>
       <c r="G3" s="16" t="inlineStr">
         <is>
-          <t>“Vidyakar”</t>
+          <t>github-actions[bot]</t>
         </is>
       </c>
       <c r="H3" s="16" t="inlineStr">
         <is>
-          <t>2026-04-10T16:02:48Z</t>
+          <t>2026-04-10T16:37:21Z</t>
         </is>
       </c>
       <c r="I3" s="16" t="inlineStr">
@@ -1088,34 +1088,12 @@
       <c r="M3" s="16" t="inlineStr"/>
       <c r="N3" s="16" t="inlineStr"/>
       <c r="O3" s="16" t="inlineStr"/>
-      <c r="P3" s="16" t="inlineStr">
-        <is>
-          <t>GitHub Activity Report</t>
-        </is>
-      </c>
-      <c r="Q3" s="16" t="n">
-        <v>24252121271</v>
-      </c>
-      <c r="R3" s="16" t="inlineStr">
-        <is>
-          <t>push</t>
-        </is>
-      </c>
-      <c r="S3" s="16" t="inlineStr">
-        <is>
-          <t>2026-04-10T16:04:46Z</t>
-        </is>
-      </c>
-      <c r="T3" s="16" t="inlineStr">
-        <is>
-          <t>completed</t>
-        </is>
-      </c>
-      <c r="U3" s="17" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
+      <c r="P3" s="16" t="inlineStr"/>
+      <c r="Q3" s="16" t="inlineStr"/>
+      <c r="R3" s="16" t="inlineStr"/>
+      <c r="S3" s="16" t="inlineStr"/>
+      <c r="T3" s="16" t="inlineStr"/>
+      <c r="U3" s="16" t="inlineStr"/>
       <c r="V3" s="16" t="inlineStr"/>
       <c r="W3" s="16" t="inlineStr"/>
       <c r="X3" s="16" t="inlineStr"/>
@@ -1123,710 +1101,732 @@
       <c r="Z3" s="16" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="16" t="inlineStr">
-        <is>
-          <t>git-report</t>
-        </is>
-      </c>
-      <c r="B4" s="16" t="inlineStr">
-        <is>
-          <t>vidyakar-whitedev</t>
-        </is>
-      </c>
-      <c r="C4" s="16" t="inlineStr">
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>git-report</t>
+        </is>
+      </c>
+      <c r="B4" s="17" t="inlineStr">
+        <is>
+          <t>vidyakar-whitedev</t>
+        </is>
+      </c>
+      <c r="C4" s="17" t="inlineStr">
         <is>
           <t>public</t>
         </is>
       </c>
-      <c r="D4" s="16" t="inlineStr">
+      <c r="D4" s="17" t="inlineStr">
         <is>
           <t>main</t>
         </is>
       </c>
-      <c r="E4" s="16" t="inlineStr">
+      <c r="E4" s="17" t="inlineStr">
+        <is>
+          <t>93bdf4123cc644f621cecd131589bff39d5376fe</t>
+        </is>
+      </c>
+      <c r="F4" s="17" t="inlineStr">
+        <is>
+          <t>test-249</t>
+        </is>
+      </c>
+      <c r="G4" s="17" t="inlineStr">
+        <is>
+          <t>“Vidyakar”</t>
+        </is>
+      </c>
+      <c r="H4" s="17" t="inlineStr">
+        <is>
+          <t>2026-04-10T16:36:38Z</t>
+        </is>
+      </c>
+      <c r="I4" s="17" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="J4" s="17" t="inlineStr"/>
+      <c r="K4" s="17" t="inlineStr"/>
+      <c r="L4" s="17" t="inlineStr"/>
+      <c r="M4" s="17" t="inlineStr"/>
+      <c r="N4" s="17" t="inlineStr"/>
+      <c r="O4" s="17" t="inlineStr"/>
+      <c r="P4" s="17" t="inlineStr">
+        <is>
+          <t>GitHub Activity Report</t>
+        </is>
+      </c>
+      <c r="Q4" s="17" t="n">
+        <v>24253439879</v>
+      </c>
+      <c r="R4" s="17" t="inlineStr">
+        <is>
+          <t>push</t>
+        </is>
+      </c>
+      <c r="S4" s="17" t="inlineStr">
+        <is>
+          <t>2026-04-10T16:36:56Z</t>
+        </is>
+      </c>
+      <c r="T4" s="17" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="U4" s="18" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="V4" s="17" t="inlineStr"/>
+      <c r="W4" s="17" t="inlineStr"/>
+      <c r="X4" s="17" t="inlineStr"/>
+      <c r="Y4" s="17" t="inlineStr"/>
+      <c r="Z4" s="17" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="17" t="inlineStr">
+        <is>
+          <t>git-report</t>
+        </is>
+      </c>
+      <c r="B5" s="17" t="inlineStr">
+        <is>
+          <t>vidyakar-whitedev</t>
+        </is>
+      </c>
+      <c r="C5" s="17" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="D5" s="17" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E5" s="17" t="inlineStr">
+        <is>
+          <t>b3ea79ed073ed633f20c5321bc134cc65896c901</t>
+        </is>
+      </c>
+      <c r="F5" s="17" t="inlineStr">
+        <is>
+          <t>test-209</t>
+        </is>
+      </c>
+      <c r="G5" s="17" t="inlineStr">
+        <is>
+          <t>“Vidyakar”</t>
+        </is>
+      </c>
+      <c r="H5" s="17" t="inlineStr">
+        <is>
+          <t>2026-04-10T16:02:48Z</t>
+        </is>
+      </c>
+      <c r="I5" s="17" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="J5" s="17" t="inlineStr"/>
+      <c r="K5" s="17" t="inlineStr"/>
+      <c r="L5" s="17" t="inlineStr"/>
+      <c r="M5" s="17" t="inlineStr"/>
+      <c r="N5" s="17" t="inlineStr"/>
+      <c r="O5" s="17" t="inlineStr"/>
+      <c r="P5" s="17" t="inlineStr">
+        <is>
+          <t>GitHub Activity Report</t>
+        </is>
+      </c>
+      <c r="Q5" s="17" t="n">
+        <v>24252121271</v>
+      </c>
+      <c r="R5" s="17" t="inlineStr">
+        <is>
+          <t>push</t>
+        </is>
+      </c>
+      <c r="S5" s="17" t="inlineStr">
+        <is>
+          <t>2026-04-10T16:04:46Z</t>
+        </is>
+      </c>
+      <c r="T5" s="17" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="U5" s="18" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="V5" s="17" t="inlineStr"/>
+      <c r="W5" s="17" t="inlineStr"/>
+      <c r="X5" s="17" t="inlineStr"/>
+      <c r="Y5" s="17" t="inlineStr"/>
+      <c r="Z5" s="17" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>git-report</t>
+        </is>
+      </c>
+      <c r="B6" s="17" t="inlineStr">
+        <is>
+          <t>vidyakar-whitedev</t>
+        </is>
+      </c>
+      <c r="C6" s="17" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="D6" s="17" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E6" s="17" t="inlineStr">
         <is>
           <t>25126c83583917e6acf1c55b3b79659ece2e2368</t>
         </is>
       </c>
-      <c r="F4" s="16" t="inlineStr">
+      <c r="F6" s="17" t="inlineStr">
         <is>
           <t>test-201</t>
         </is>
       </c>
-      <c r="G4" s="16" t="inlineStr">
+      <c r="G6" s="17" t="inlineStr">
         <is>
           <t>“Vidyakar”</t>
         </is>
       </c>
-      <c r="H4" s="16" t="inlineStr">
+      <c r="H6" s="17" t="inlineStr">
         <is>
           <t>2026-04-10T15:26:42Z</t>
         </is>
       </c>
-      <c r="I4" s="16" t="inlineStr">
+      <c r="I6" s="17" t="inlineStr">
         <is>
           <t>main</t>
         </is>
       </c>
-      <c r="J4" s="16" t="inlineStr"/>
-      <c r="K4" s="16" t="inlineStr"/>
-      <c r="L4" s="16" t="inlineStr"/>
-      <c r="M4" s="16" t="inlineStr"/>
-      <c r="N4" s="16" t="inlineStr"/>
-      <c r="O4" s="16" t="inlineStr"/>
-      <c r="P4" s="16" t="inlineStr">
+      <c r="J6" s="17" t="inlineStr"/>
+      <c r="K6" s="17" t="inlineStr"/>
+      <c r="L6" s="17" t="inlineStr"/>
+      <c r="M6" s="17" t="inlineStr"/>
+      <c r="N6" s="17" t="inlineStr"/>
+      <c r="O6" s="17" t="inlineStr"/>
+      <c r="P6" s="17" t="inlineStr">
         <is>
           <t>GitHub Activity Report</t>
         </is>
       </c>
-      <c r="Q4" s="16" t="n">
+      <c r="Q6" s="17" t="n">
         <v>24250548345</v>
       </c>
-      <c r="R4" s="16" t="inlineStr">
+      <c r="R6" s="17" t="inlineStr">
         <is>
           <t>push</t>
         </is>
       </c>
-      <c r="S4" s="16" t="inlineStr">
+      <c r="S6" s="17" t="inlineStr">
         <is>
           <t>2026-04-10T15:27:44Z</t>
         </is>
       </c>
-      <c r="T4" s="16" t="inlineStr">
+      <c r="T6" s="17" t="inlineStr">
         <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="U4" s="17" t="inlineStr">
+      <c r="U6" s="18" t="inlineStr">
         <is>
           <t>success</t>
         </is>
       </c>
-      <c r="V4" s="16" t="inlineStr"/>
-      <c r="W4" s="16" t="inlineStr"/>
-      <c r="X4" s="16" t="inlineStr"/>
-      <c r="Y4" s="16" t="inlineStr"/>
-      <c r="Z4" s="16" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="18" t="inlineStr">
-        <is>
-          <t>git-report</t>
-        </is>
-      </c>
-      <c r="B5" s="18" t="inlineStr">
-        <is>
-          <t>vidyakar-whitedev</t>
-        </is>
-      </c>
-      <c r="C5" s="18" t="inlineStr">
+      <c r="V6" s="17" t="inlineStr"/>
+      <c r="W6" s="17" t="inlineStr"/>
+      <c r="X6" s="17" t="inlineStr"/>
+      <c r="Y6" s="17" t="inlineStr"/>
+      <c r="Z6" s="17" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="16" t="inlineStr">
+        <is>
+          <t>git-report</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>vidyakar-whitedev</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
         <is>
           <t>public</t>
         </is>
       </c>
-      <c r="D5" s="18" t="inlineStr">
+      <c r="D7" s="16" t="inlineStr">
         <is>
           <t>main</t>
         </is>
       </c>
-      <c r="E5" s="18" t="inlineStr">
+      <c r="E7" s="16" t="inlineStr">
         <is>
           <t>9e3c7f0f229aff7c1984cec897ef7c43ff34c5e8</t>
         </is>
       </c>
-      <c r="F5" s="18" t="inlineStr">
+      <c r="F7" s="16" t="inlineStr">
         <is>
           <t>chore: update activity report [2026-04-10 15:17 UTC] via push (run 24250086438)</t>
         </is>
       </c>
-      <c r="G5" s="18" t="inlineStr">
+      <c r="G7" s="16" t="inlineStr">
         <is>
           <t>github-actions[bot]</t>
         </is>
       </c>
-      <c r="H5" s="18" t="inlineStr">
+      <c r="H7" s="16" t="inlineStr">
         <is>
           <t>2026-04-10T15:17:35Z</t>
         </is>
       </c>
-      <c r="I5" s="18" t="inlineStr">
+      <c r="I7" s="16" t="inlineStr">
         <is>
           <t>main</t>
         </is>
       </c>
-      <c r="J5" s="18" t="inlineStr"/>
-      <c r="K5" s="18" t="inlineStr"/>
-      <c r="L5" s="18" t="inlineStr"/>
-      <c r="M5" s="18" t="inlineStr"/>
-      <c r="N5" s="18" t="inlineStr"/>
-      <c r="O5" s="18" t="inlineStr"/>
-      <c r="P5" s="18" t="inlineStr"/>
-      <c r="Q5" s="18" t="inlineStr"/>
-      <c r="R5" s="18" t="inlineStr"/>
-      <c r="S5" s="18" t="inlineStr"/>
-      <c r="T5" s="18" t="inlineStr"/>
-      <c r="U5" s="18" t="inlineStr"/>
-      <c r="V5" s="18" t="inlineStr"/>
-      <c r="W5" s="18" t="inlineStr"/>
-      <c r="X5" s="18" t="inlineStr"/>
-      <c r="Y5" s="18" t="inlineStr"/>
-      <c r="Z5" s="18" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="19" t="inlineStr">
-        <is>
-          <t>git-report</t>
-        </is>
-      </c>
-      <c r="B6" s="19" t="inlineStr">
-        <is>
-          <t>vidyakar-whitedev</t>
-        </is>
-      </c>
-      <c r="C6" s="19" t="inlineStr">
+      <c r="J7" s="16" t="inlineStr"/>
+      <c r="K7" s="16" t="inlineStr"/>
+      <c r="L7" s="16" t="inlineStr"/>
+      <c r="M7" s="16" t="inlineStr"/>
+      <c r="N7" s="16" t="inlineStr"/>
+      <c r="O7" s="16" t="inlineStr"/>
+      <c r="P7" s="16" t="inlineStr"/>
+      <c r="Q7" s="16" t="inlineStr"/>
+      <c r="R7" s="16" t="inlineStr"/>
+      <c r="S7" s="16" t="inlineStr"/>
+      <c r="T7" s="16" t="inlineStr"/>
+      <c r="U7" s="16" t="inlineStr"/>
+      <c r="V7" s="16" t="inlineStr"/>
+      <c r="W7" s="16" t="inlineStr"/>
+      <c r="X7" s="16" t="inlineStr"/>
+      <c r="Y7" s="16" t="inlineStr"/>
+      <c r="Z7" s="16" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="19" t="inlineStr">
+        <is>
+          <t>git-report</t>
+        </is>
+      </c>
+      <c r="B8" s="19" t="inlineStr">
+        <is>
+          <t>vidyakar-whitedev</t>
+        </is>
+      </c>
+      <c r="C8" s="19" t="inlineStr">
         <is>
           <t>public</t>
         </is>
       </c>
-      <c r="D6" s="19" t="inlineStr">
+      <c r="D8" s="19" t="inlineStr">
         <is>
           <t>main</t>
         </is>
       </c>
-      <c r="E6" s="19" t="inlineStr">
+      <c r="E8" s="19" t="inlineStr">
         <is>
           <t>0bf36a490d78a4819928a11161d34bda33e4f337</t>
         </is>
       </c>
-      <c r="F6" s="19" t="inlineStr">
+      <c r="F8" s="19" t="inlineStr">
         <is>
           <t>test-200</t>
         </is>
       </c>
-      <c r="G6" s="19" t="inlineStr">
+      <c r="G8" s="19" t="inlineStr">
         <is>
           <t>“Vidyakar”</t>
         </is>
       </c>
-      <c r="H6" s="19" t="inlineStr">
+      <c r="H8" s="19" t="inlineStr">
         <is>
           <t>2026-04-10T15:16:43Z</t>
         </is>
       </c>
-      <c r="I6" s="19" t="inlineStr">
+      <c r="I8" s="19" t="inlineStr">
         <is>
           <t>main</t>
         </is>
       </c>
-      <c r="J6" s="19" t="inlineStr"/>
-      <c r="K6" s="19" t="inlineStr"/>
-      <c r="L6" s="19" t="inlineStr"/>
-      <c r="M6" s="19" t="inlineStr"/>
-      <c r="N6" s="19" t="inlineStr"/>
-      <c r="O6" s="19" t="inlineStr"/>
-      <c r="P6" s="19" t="inlineStr">
+      <c r="J8" s="19" t="inlineStr"/>
+      <c r="K8" s="19" t="inlineStr"/>
+      <c r="L8" s="19" t="inlineStr"/>
+      <c r="M8" s="19" t="inlineStr"/>
+      <c r="N8" s="19" t="inlineStr"/>
+      <c r="O8" s="19" t="inlineStr"/>
+      <c r="P8" s="19" t="inlineStr">
         <is>
           <t>GitHub Activity Report</t>
         </is>
       </c>
-      <c r="Q6" s="19" t="n">
+      <c r="Q8" s="19" t="n">
         <v>24250086438</v>
       </c>
-      <c r="R6" s="19" t="inlineStr">
+      <c r="R8" s="19" t="inlineStr">
         <is>
           <t>push</t>
         </is>
       </c>
-      <c r="S6" s="19" t="inlineStr">
+      <c r="S8" s="19" t="inlineStr">
         <is>
           <t>2026-04-10T15:18:50Z</t>
         </is>
       </c>
-      <c r="T6" s="19" t="inlineStr">
+      <c r="T8" s="19" t="inlineStr">
         <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="U6" s="20" t="inlineStr">
+      <c r="U8" s="20" t="inlineStr">
         <is>
           <t>failure</t>
         </is>
       </c>
-      <c r="V6" s="19" t="inlineStr">
+      <c r="V8" s="19" t="inlineStr">
         <is>
           <t>Job 'generate_report' step 'Commit and push report to repository' failed — 2026-04-10T15:19:10.4298620Z 15:19:10  WARNING   WORKFLOW FAILURE in vidyakar-whitedev/git-report  (Run ID: 24030846379)</t>
         </is>
       </c>
-      <c r="W6" s="19" t="inlineStr">
+      <c r="W8" s="19" t="inlineStr">
         <is>
           <t>generate_report</t>
         </is>
       </c>
-      <c r="X6" s="19" t="inlineStr">
+      <c r="X8" s="19" t="inlineStr">
         <is>
           <t>Commit and push report to repository</t>
         </is>
       </c>
-      <c r="Y6" s="19" t="inlineStr">
+      <c r="Y8" s="19" t="inlineStr">
         <is>
           <t>Line 19</t>
         </is>
       </c>
-      <c r="Z6" s="19" t="inlineStr">
+      <c r="Z8" s="19" t="inlineStr">
         <is>
           <t>Auth/permission error — verify GH_PAT scopes and that repository secrets are correctly configured.</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="18" t="inlineStr">
-        <is>
-          <t>git-report</t>
-        </is>
-      </c>
-      <c r="B7" s="18" t="inlineStr">
-        <is>
-          <t>vidyakar-whitedev</t>
-        </is>
-      </c>
-      <c r="C7" s="18" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="16" t="inlineStr">
+        <is>
+          <t>git-report</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>vidyakar-whitedev</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
         <is>
           <t>public</t>
         </is>
       </c>
-      <c r="D7" s="18" t="inlineStr">
+      <c r="D9" s="16" t="inlineStr">
         <is>
           <t>main</t>
         </is>
       </c>
-      <c r="E7" s="18" t="inlineStr">
+      <c r="E9" s="16" t="inlineStr">
         <is>
           <t>4744a63d54822fd75d284791aa8b6524acb33646</t>
         </is>
       </c>
-      <c r="F7" s="18" t="inlineStr">
+      <c r="F9" s="16" t="inlineStr">
         <is>
           <t>chore: update activity report [2026-04-10 14:39 UTC] via push (run 24248391662)</t>
         </is>
       </c>
-      <c r="G7" s="18" t="inlineStr">
+      <c r="G9" s="16" t="inlineStr">
         <is>
           <t>github-actions[bot]</t>
         </is>
       </c>
-      <c r="H7" s="18" t="inlineStr">
+      <c r="H9" s="16" t="inlineStr">
         <is>
           <t>2026-04-10T14:39:22Z</t>
         </is>
       </c>
-      <c r="I7" s="18" t="inlineStr">
+      <c r="I9" s="16" t="inlineStr">
         <is>
           <t>main</t>
         </is>
       </c>
-      <c r="J7" s="18" t="inlineStr"/>
-      <c r="K7" s="18" t="inlineStr"/>
-      <c r="L7" s="18" t="inlineStr"/>
-      <c r="M7" s="18" t="inlineStr"/>
-      <c r="N7" s="18" t="inlineStr"/>
-      <c r="O7" s="18" t="inlineStr"/>
-      <c r="P7" s="18" t="inlineStr"/>
-      <c r="Q7" s="18" t="inlineStr"/>
-      <c r="R7" s="18" t="inlineStr"/>
-      <c r="S7" s="18" t="inlineStr"/>
-      <c r="T7" s="18" t="inlineStr"/>
-      <c r="U7" s="18" t="inlineStr"/>
-      <c r="V7" s="18" t="inlineStr"/>
-      <c r="W7" s="18" t="inlineStr"/>
-      <c r="X7" s="18" t="inlineStr"/>
-      <c r="Y7" s="18" t="inlineStr"/>
-      <c r="Z7" s="18" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="16" t="inlineStr">
-        <is>
-          <t>git-report</t>
-        </is>
-      </c>
-      <c r="B8" s="16" t="inlineStr">
-        <is>
-          <t>vidyakar-whitedev</t>
-        </is>
-      </c>
-      <c r="C8" s="16" t="inlineStr">
+      <c r="J9" s="16" t="inlineStr"/>
+      <c r="K9" s="16" t="inlineStr"/>
+      <c r="L9" s="16" t="inlineStr"/>
+      <c r="M9" s="16" t="inlineStr"/>
+      <c r="N9" s="16" t="inlineStr"/>
+      <c r="O9" s="16" t="inlineStr"/>
+      <c r="P9" s="16" t="inlineStr"/>
+      <c r="Q9" s="16" t="inlineStr"/>
+      <c r="R9" s="16" t="inlineStr"/>
+      <c r="S9" s="16" t="inlineStr"/>
+      <c r="T9" s="16" t="inlineStr"/>
+      <c r="U9" s="16" t="inlineStr"/>
+      <c r="V9" s="16" t="inlineStr"/>
+      <c r="W9" s="16" t="inlineStr"/>
+      <c r="X9" s="16" t="inlineStr"/>
+      <c r="Y9" s="16" t="inlineStr"/>
+      <c r="Z9" s="16" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>git-report</t>
+        </is>
+      </c>
+      <c r="B10" s="17" t="inlineStr">
+        <is>
+          <t>vidyakar-whitedev</t>
+        </is>
+      </c>
+      <c r="C10" s="17" t="inlineStr">
         <is>
           <t>public</t>
         </is>
       </c>
-      <c r="D8" s="16" t="inlineStr">
+      <c r="D10" s="17" t="inlineStr">
         <is>
           <t>main</t>
         </is>
       </c>
-      <c r="E8" s="16" t="inlineStr">
+      <c r="E10" s="17" t="inlineStr">
         <is>
           <t>408ddd043c24815f4498a813c6ca81c4e9688b9b</t>
         </is>
       </c>
-      <c r="F8" s="16" t="inlineStr">
+      <c r="F10" s="17" t="inlineStr">
         <is>
           <t>test-198</t>
         </is>
       </c>
-      <c r="G8" s="16" t="inlineStr">
+      <c r="G10" s="17" t="inlineStr">
         <is>
           <t>“Vidyakar”</t>
         </is>
       </c>
-      <c r="H8" s="16" t="inlineStr">
+      <c r="H10" s="17" t="inlineStr">
         <is>
           <t>2026-04-10T14:38:25Z</t>
         </is>
       </c>
-      <c r="I8" s="16" t="inlineStr">
+      <c r="I10" s="17" t="inlineStr">
         <is>
           <t>main</t>
         </is>
       </c>
-      <c r="J8" s="16" t="inlineStr"/>
-      <c r="K8" s="16" t="inlineStr"/>
-      <c r="L8" s="16" t="inlineStr"/>
-      <c r="M8" s="16" t="inlineStr"/>
-      <c r="N8" s="16" t="inlineStr"/>
-      <c r="O8" s="16" t="inlineStr"/>
-      <c r="P8" s="16" t="inlineStr">
+      <c r="J10" s="17" t="inlineStr"/>
+      <c r="K10" s="17" t="inlineStr"/>
+      <c r="L10" s="17" t="inlineStr"/>
+      <c r="M10" s="17" t="inlineStr"/>
+      <c r="N10" s="17" t="inlineStr"/>
+      <c r="O10" s="17" t="inlineStr"/>
+      <c r="P10" s="17" t="inlineStr">
         <is>
           <t>GitHub Activity Report</t>
         </is>
       </c>
-      <c r="Q8" s="16" t="n">
+      <c r="Q10" s="17" t="n">
         <v>24248391662</v>
       </c>
-      <c r="R8" s="16" t="inlineStr">
+      <c r="R10" s="17" t="inlineStr">
         <is>
           <t>push</t>
         </is>
       </c>
-      <c r="S8" s="16" t="inlineStr">
+      <c r="S10" s="17" t="inlineStr">
         <is>
           <t>2026-04-10T14:38:48Z</t>
         </is>
       </c>
-      <c r="T8" s="16" t="inlineStr">
+      <c r="T10" s="17" t="inlineStr">
         <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="U8" s="17" t="inlineStr">
+      <c r="U10" s="18" t="inlineStr">
         <is>
           <t>success</t>
         </is>
       </c>
-      <c r="V8" s="16" t="inlineStr"/>
-      <c r="W8" s="16" t="inlineStr"/>
-      <c r="X8" s="16" t="inlineStr"/>
-      <c r="Y8" s="16" t="inlineStr"/>
-      <c r="Z8" s="16" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="18" t="inlineStr">
-        <is>
-          <t>git-report</t>
-        </is>
-      </c>
-      <c r="B9" s="18" t="inlineStr">
-        <is>
-          <t>vidyakar-whitedev</t>
-        </is>
-      </c>
-      <c r="C9" s="18" t="inlineStr">
+      <c r="V10" s="17" t="inlineStr"/>
+      <c r="W10" s="17" t="inlineStr"/>
+      <c r="X10" s="17" t="inlineStr"/>
+      <c r="Y10" s="17" t="inlineStr"/>
+      <c r="Z10" s="17" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="16" t="inlineStr">
+        <is>
+          <t>git-report</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>vidyakar-whitedev</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
         <is>
           <t>public</t>
         </is>
       </c>
-      <c r="D9" s="18" t="inlineStr">
+      <c r="D11" s="16" t="inlineStr">
         <is>
           <t>main</t>
         </is>
       </c>
-      <c r="E9" s="18" t="inlineStr">
+      <c r="E11" s="16" t="inlineStr">
         <is>
           <t>37f60b0c23d45eef199630a384945ef73970b8d7</t>
         </is>
       </c>
-      <c r="F9" s="18" t="inlineStr">
+      <c r="F11" s="16" t="inlineStr">
         <is>
           <t>chore: update activity report [2026-04-10 09:44 UTC] via push (run 24236872105)</t>
         </is>
       </c>
-      <c r="G9" s="18" t="inlineStr">
+      <c r="G11" s="16" t="inlineStr">
         <is>
           <t>github-actions[bot]</t>
         </is>
       </c>
-      <c r="H9" s="18" t="inlineStr">
+      <c r="H11" s="16" t="inlineStr">
         <is>
           <t>2026-04-10T09:44:03Z</t>
         </is>
       </c>
-      <c r="I9" s="18" t="inlineStr">
+      <c r="I11" s="16" t="inlineStr">
         <is>
           <t>main</t>
         </is>
       </c>
-      <c r="J9" s="18" t="inlineStr"/>
-      <c r="K9" s="18" t="inlineStr"/>
-      <c r="L9" s="18" t="inlineStr"/>
-      <c r="M9" s="18" t="inlineStr"/>
-      <c r="N9" s="18" t="inlineStr"/>
-      <c r="O9" s="18" t="inlineStr"/>
-      <c r="P9" s="18" t="inlineStr"/>
-      <c r="Q9" s="18" t="inlineStr"/>
-      <c r="R9" s="18" t="inlineStr"/>
-      <c r="S9" s="18" t="inlineStr"/>
-      <c r="T9" s="18" t="inlineStr"/>
-      <c r="U9" s="18" t="inlineStr"/>
-      <c r="V9" s="18" t="inlineStr"/>
-      <c r="W9" s="18" t="inlineStr"/>
-      <c r="X9" s="18" t="inlineStr"/>
-      <c r="Y9" s="18" t="inlineStr"/>
-      <c r="Z9" s="18" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="16" t="inlineStr">
-        <is>
-          <t>git-report</t>
-        </is>
-      </c>
-      <c r="B10" s="16" t="inlineStr">
-        <is>
-          <t>vidyakar-whitedev</t>
-        </is>
-      </c>
-      <c r="C10" s="16" t="inlineStr">
+      <c r="J11" s="16" t="inlineStr"/>
+      <c r="K11" s="16" t="inlineStr"/>
+      <c r="L11" s="16" t="inlineStr"/>
+      <c r="M11" s="16" t="inlineStr"/>
+      <c r="N11" s="16" t="inlineStr"/>
+      <c r="O11" s="16" t="inlineStr"/>
+      <c r="P11" s="16" t="inlineStr"/>
+      <c r="Q11" s="16" t="inlineStr"/>
+      <c r="R11" s="16" t="inlineStr"/>
+      <c r="S11" s="16" t="inlineStr"/>
+      <c r="T11" s="16" t="inlineStr"/>
+      <c r="U11" s="16" t="inlineStr"/>
+      <c r="V11" s="16" t="inlineStr"/>
+      <c r="W11" s="16" t="inlineStr"/>
+      <c r="X11" s="16" t="inlineStr"/>
+      <c r="Y11" s="16" t="inlineStr"/>
+      <c r="Z11" s="16" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>git-report</t>
+        </is>
+      </c>
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t>vidyakar-whitedev</t>
+        </is>
+      </c>
+      <c r="C12" s="17" t="inlineStr">
         <is>
           <t>public</t>
         </is>
       </c>
-      <c r="D10" s="16" t="inlineStr">
+      <c r="D12" s="17" t="inlineStr">
         <is>
           <t>main</t>
         </is>
       </c>
-      <c r="E10" s="16" t="inlineStr">
+      <c r="E12" s="17" t="inlineStr">
         <is>
           <t>aac0b4a033d6b371042ec3f99a213aa53e5d925f</t>
         </is>
       </c>
-      <c r="F10" s="16" t="inlineStr">
+      <c r="F12" s="17" t="inlineStr">
         <is>
           <t>test-198</t>
         </is>
       </c>
-      <c r="G10" s="16" t="inlineStr">
+      <c r="G12" s="17" t="inlineStr">
         <is>
           <t>“Vidyakar”</t>
         </is>
       </c>
-      <c r="H10" s="16" t="inlineStr">
+      <c r="H12" s="17" t="inlineStr">
         <is>
           <t>2026-04-10T09:40:50Z</t>
         </is>
       </c>
-      <c r="I10" s="16" t="inlineStr">
+      <c r="I12" s="17" t="inlineStr">
         <is>
           <t>main</t>
         </is>
       </c>
-      <c r="J10" s="16" t="inlineStr"/>
-      <c r="K10" s="16" t="inlineStr"/>
-      <c r="L10" s="16" t="inlineStr"/>
-      <c r="M10" s="16" t="inlineStr"/>
-      <c r="N10" s="16" t="inlineStr"/>
-      <c r="O10" s="16" t="inlineStr"/>
-      <c r="P10" s="16" t="inlineStr">
+      <c r="J12" s="17" t="inlineStr"/>
+      <c r="K12" s="17" t="inlineStr"/>
+      <c r="L12" s="17" t="inlineStr"/>
+      <c r="M12" s="17" t="inlineStr"/>
+      <c r="N12" s="17" t="inlineStr"/>
+      <c r="O12" s="17" t="inlineStr"/>
+      <c r="P12" s="17" t="inlineStr">
         <is>
           <t>GitHub Activity Report</t>
         </is>
       </c>
-      <c r="Q10" s="16" t="n">
+      <c r="Q12" s="17" t="n">
         <v>24236872105</v>
       </c>
-      <c r="R10" s="16" t="inlineStr">
+      <c r="R12" s="17" t="inlineStr">
         <is>
           <t>push</t>
         </is>
       </c>
-      <c r="S10" s="16" t="inlineStr">
+      <c r="S12" s="17" t="inlineStr">
         <is>
           <t>2026-04-10T09:43:38Z</t>
         </is>
       </c>
-      <c r="T10" s="16" t="inlineStr">
+      <c r="T12" s="17" t="inlineStr">
         <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="U10" s="17" t="inlineStr">
+      <c r="U12" s="18" t="inlineStr">
         <is>
           <t>success</t>
         </is>
       </c>
-      <c r="V10" s="16" t="inlineStr"/>
-      <c r="W10" s="16" t="inlineStr"/>
-      <c r="X10" s="16" t="inlineStr"/>
-      <c r="Y10" s="16" t="inlineStr"/>
-      <c r="Z10" s="16" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="18" t="inlineStr">
-        <is>
-          <t>git-report</t>
-        </is>
-      </c>
-      <c r="B11" s="18" t="inlineStr">
-        <is>
-          <t>vidyakar-whitedev</t>
-        </is>
-      </c>
-      <c r="C11" s="18" t="inlineStr">
-        <is>
-          <t>public</t>
-        </is>
-      </c>
-      <c r="D11" s="18" t="inlineStr">
-        <is>
-          <t>main</t>
-        </is>
-      </c>
-      <c r="E11" s="18" t="inlineStr">
-        <is>
-          <t>19b0e6e1eadc37093a80d5aa3b43d47cf52cc739</t>
-        </is>
-      </c>
-      <c r="F11" s="18" t="inlineStr">
-        <is>
-          <t>chore: update activity report [2026-04-10 09:36 UTC] via push (run 24236579665)</t>
-        </is>
-      </c>
-      <c r="G11" s="18" t="inlineStr">
-        <is>
-          <t>github-actions[bot]</t>
-        </is>
-      </c>
-      <c r="H11" s="18" t="inlineStr">
-        <is>
-          <t>2026-04-10T09:36:36Z</t>
-        </is>
-      </c>
-      <c r="I11" s="18" t="inlineStr">
-        <is>
-          <t>main</t>
-        </is>
-      </c>
-      <c r="J11" s="18" t="inlineStr"/>
-      <c r="K11" s="18" t="inlineStr"/>
-      <c r="L11" s="18" t="inlineStr"/>
-      <c r="M11" s="18" t="inlineStr"/>
-      <c r="N11" s="18" t="inlineStr"/>
-      <c r="O11" s="18" t="inlineStr"/>
-      <c r="P11" s="18" t="inlineStr"/>
-      <c r="Q11" s="18" t="inlineStr"/>
-      <c r="R11" s="18" t="inlineStr"/>
-      <c r="S11" s="18" t="inlineStr"/>
-      <c r="T11" s="18" t="inlineStr"/>
-      <c r="U11" s="18" t="inlineStr"/>
-      <c r="V11" s="18" t="inlineStr"/>
-      <c r="W11" s="18" t="inlineStr"/>
-      <c r="X11" s="18" t="inlineStr"/>
-      <c r="Y11" s="18" t="inlineStr"/>
-      <c r="Z11" s="18" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="16" t="inlineStr">
-        <is>
-          <t>git-report</t>
-        </is>
-      </c>
-      <c r="B12" s="16" t="inlineStr">
-        <is>
-          <t>vidyakar-whitedev</t>
-        </is>
-      </c>
-      <c r="C12" s="16" t="inlineStr">
-        <is>
-          <t>public</t>
-        </is>
-      </c>
-      <c r="D12" s="16" t="inlineStr">
-        <is>
-          <t>main</t>
-        </is>
-      </c>
-      <c r="E12" s="16" t="inlineStr">
-        <is>
-          <t>4246e5f5bdd0c663224514d45c37457253e6806b</t>
-        </is>
-      </c>
-      <c r="F12" s="16" t="inlineStr">
-        <is>
-          <t>test-13</t>
-        </is>
-      </c>
-      <c r="G12" s="16" t="inlineStr">
-        <is>
-          <t>“Vidyakar”</t>
-        </is>
-      </c>
-      <c r="H12" s="16" t="inlineStr">
-        <is>
-          <t>2026-04-10T09:35:54Z</t>
-        </is>
-      </c>
-      <c r="I12" s="16" t="inlineStr">
-        <is>
-          <t>main</t>
-        </is>
-      </c>
-      <c r="J12" s="16" t="inlineStr"/>
-      <c r="K12" s="16" t="inlineStr"/>
-      <c r="L12" s="16" t="inlineStr"/>
-      <c r="M12" s="16" t="inlineStr"/>
-      <c r="N12" s="16" t="inlineStr"/>
-      <c r="O12" s="16" t="inlineStr"/>
-      <c r="P12" s="16" t="inlineStr">
-        <is>
-          <t>GitHub Activity Report</t>
-        </is>
-      </c>
-      <c r="Q12" s="16" t="n">
-        <v>24236579665</v>
-      </c>
-      <c r="R12" s="16" t="inlineStr">
-        <is>
-          <t>push</t>
-        </is>
-      </c>
-      <c r="S12" s="16" t="inlineStr">
-        <is>
-          <t>2026-04-10T09:36:01Z</t>
-        </is>
-      </c>
-      <c r="T12" s="16" t="inlineStr">
-        <is>
-          <t>completed</t>
-        </is>
-      </c>
-      <c r="U12" s="17" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
-      <c r="V12" s="16" t="inlineStr"/>
-      <c r="W12" s="16" t="inlineStr"/>
-      <c r="X12" s="16" t="inlineStr"/>
-      <c r="Y12" s="16" t="inlineStr"/>
-      <c r="Z12" s="16" t="inlineStr"/>
+      <c r="V12" s="17" t="inlineStr"/>
+      <c r="W12" s="17" t="inlineStr"/>
+      <c r="X12" s="17" t="inlineStr"/>
+      <c r="Y12" s="17" t="inlineStr"/>
+      <c r="Z12" s="17" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="16" t="inlineStr">
@@ -1851,22 +1851,22 @@
       </c>
       <c r="E13" s="16" t="inlineStr">
         <is>
-          <t>ff12234265b7ed9747283a1b59735ea5ddda19b5</t>
+          <t>19b0e6e1eadc37093a80d5aa3b43d47cf52cc739</t>
         </is>
       </c>
       <c r="F13" s="16" t="inlineStr">
         <is>
-          <t>test-12</t>
+          <t>chore: update activity report [2026-04-10 09:36 UTC] via push (run 24236579665)</t>
         </is>
       </c>
       <c r="G13" s="16" t="inlineStr">
         <is>
-          <t>“Vidyakar”</t>
+          <t>github-actions[bot]</t>
         </is>
       </c>
       <c r="H13" s="16" t="inlineStr">
         <is>
-          <t>2026-04-10T09:21:24Z</t>
+          <t>2026-04-10T09:36:36Z</t>
         </is>
       </c>
       <c r="I13" s="16" t="inlineStr">
@@ -1880,34 +1880,12 @@
       <c r="M13" s="16" t="inlineStr"/>
       <c r="N13" s="16" t="inlineStr"/>
       <c r="O13" s="16" t="inlineStr"/>
-      <c r="P13" s="16" t="inlineStr">
-        <is>
-          <t>GitHub Activity Report</t>
-        </is>
-      </c>
-      <c r="Q13" s="16" t="n">
-        <v>24236015736</v>
-      </c>
-      <c r="R13" s="16" t="inlineStr">
-        <is>
-          <t>push</t>
-        </is>
-      </c>
-      <c r="S13" s="16" t="inlineStr">
-        <is>
-          <t>2026-04-10T09:21:36Z</t>
-        </is>
-      </c>
-      <c r="T13" s="16" t="inlineStr">
-        <is>
-          <t>completed</t>
-        </is>
-      </c>
-      <c r="U13" s="17" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
+      <c r="P13" s="16" t="inlineStr"/>
+      <c r="Q13" s="16" t="inlineStr"/>
+      <c r="R13" s="16" t="inlineStr"/>
+      <c r="S13" s="16" t="inlineStr"/>
+      <c r="T13" s="16" t="inlineStr"/>
+      <c r="U13" s="16" t="inlineStr"/>
       <c r="V13" s="16" t="inlineStr"/>
       <c r="W13" s="16" t="inlineStr"/>
       <c r="X13" s="16" t="inlineStr"/>
@@ -1915,732 +1893,692 @@
       <c r="Z13" s="16" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="16" t="inlineStr">
-        <is>
-          <t>git-report</t>
-        </is>
-      </c>
-      <c r="B14" s="16" t="inlineStr">
-        <is>
-          <t>vidyakar-whitedev</t>
-        </is>
-      </c>
-      <c r="C14" s="16" t="inlineStr">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>git-report</t>
+        </is>
+      </c>
+      <c r="B14" s="17" t="inlineStr">
+        <is>
+          <t>vidyakar-whitedev</t>
+        </is>
+      </c>
+      <c r="C14" s="17" t="inlineStr">
         <is>
           <t>public</t>
         </is>
       </c>
-      <c r="D14" s="16" t="inlineStr">
+      <c r="D14" s="17" t="inlineStr">
         <is>
           <t>main</t>
         </is>
       </c>
-      <c r="E14" s="16" t="inlineStr">
+      <c r="E14" s="17" t="inlineStr">
+        <is>
+          <t>4246e5f5bdd0c663224514d45c37457253e6806b</t>
+        </is>
+      </c>
+      <c r="F14" s="17" t="inlineStr">
+        <is>
+          <t>test-13</t>
+        </is>
+      </c>
+      <c r="G14" s="17" t="inlineStr">
+        <is>
+          <t>“Vidyakar”</t>
+        </is>
+      </c>
+      <c r="H14" s="17" t="inlineStr">
+        <is>
+          <t>2026-04-10T09:35:54Z</t>
+        </is>
+      </c>
+      <c r="I14" s="17" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="J14" s="17" t="inlineStr"/>
+      <c r="K14" s="17" t="inlineStr"/>
+      <c r="L14" s="17" t="inlineStr"/>
+      <c r="M14" s="17" t="inlineStr"/>
+      <c r="N14" s="17" t="inlineStr"/>
+      <c r="O14" s="17" t="inlineStr"/>
+      <c r="P14" s="17" t="inlineStr">
+        <is>
+          <t>GitHub Activity Report</t>
+        </is>
+      </c>
+      <c r="Q14" s="17" t="n">
+        <v>24236579665</v>
+      </c>
+      <c r="R14" s="17" t="inlineStr">
+        <is>
+          <t>push</t>
+        </is>
+      </c>
+      <c r="S14" s="17" t="inlineStr">
+        <is>
+          <t>2026-04-10T09:36:01Z</t>
+        </is>
+      </c>
+      <c r="T14" s="17" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="U14" s="18" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="V14" s="17" t="inlineStr"/>
+      <c r="W14" s="17" t="inlineStr"/>
+      <c r="X14" s="17" t="inlineStr"/>
+      <c r="Y14" s="17" t="inlineStr"/>
+      <c r="Z14" s="17" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="17" t="inlineStr">
+        <is>
+          <t>git-report</t>
+        </is>
+      </c>
+      <c r="B15" s="17" t="inlineStr">
+        <is>
+          <t>vidyakar-whitedev</t>
+        </is>
+      </c>
+      <c r="C15" s="17" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="D15" s="17" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E15" s="17" t="inlineStr">
+        <is>
+          <t>ff12234265b7ed9747283a1b59735ea5ddda19b5</t>
+        </is>
+      </c>
+      <c r="F15" s="17" t="inlineStr">
+        <is>
+          <t>test-12</t>
+        </is>
+      </c>
+      <c r="G15" s="17" t="inlineStr">
+        <is>
+          <t>“Vidyakar”</t>
+        </is>
+      </c>
+      <c r="H15" s="17" t="inlineStr">
+        <is>
+          <t>2026-04-10T09:21:24Z</t>
+        </is>
+      </c>
+      <c r="I15" s="17" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="J15" s="17" t="inlineStr"/>
+      <c r="K15" s="17" t="inlineStr"/>
+      <c r="L15" s="17" t="inlineStr"/>
+      <c r="M15" s="17" t="inlineStr"/>
+      <c r="N15" s="17" t="inlineStr"/>
+      <c r="O15" s="17" t="inlineStr"/>
+      <c r="P15" s="17" t="inlineStr">
+        <is>
+          <t>GitHub Activity Report</t>
+        </is>
+      </c>
+      <c r="Q15" s="17" t="n">
+        <v>24236015736</v>
+      </c>
+      <c r="R15" s="17" t="inlineStr">
+        <is>
+          <t>push</t>
+        </is>
+      </c>
+      <c r="S15" s="17" t="inlineStr">
+        <is>
+          <t>2026-04-10T09:21:36Z</t>
+        </is>
+      </c>
+      <c r="T15" s="17" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="U15" s="18" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="V15" s="17" t="inlineStr"/>
+      <c r="W15" s="17" t="inlineStr"/>
+      <c r="X15" s="17" t="inlineStr"/>
+      <c r="Y15" s="17" t="inlineStr"/>
+      <c r="Z15" s="17" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>git-report</t>
+        </is>
+      </c>
+      <c r="B16" s="17" t="inlineStr">
+        <is>
+          <t>vidyakar-whitedev</t>
+        </is>
+      </c>
+      <c r="C16" s="17" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="D16" s="17" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E16" s="17" t="inlineStr">
         <is>
           <t>75732834dd766afc090c808510eb71c7693015dd</t>
         </is>
       </c>
-      <c r="F14" s="16" t="inlineStr">
+      <c r="F16" s="17" t="inlineStr">
         <is>
           <t>test-8</t>
         </is>
       </c>
-      <c r="G14" s="16" t="inlineStr">
+      <c r="G16" s="17" t="inlineStr">
         <is>
           <t>“Vidyakar”</t>
         </is>
       </c>
-      <c r="H14" s="16" t="inlineStr">
+      <c r="H16" s="17" t="inlineStr">
         <is>
           <t>2026-04-10T08:35:13Z</t>
         </is>
       </c>
-      <c r="I14" s="16" t="inlineStr">
+      <c r="I16" s="17" t="inlineStr">
         <is>
           <t>main</t>
         </is>
       </c>
-      <c r="J14" s="16" t="inlineStr"/>
-      <c r="K14" s="16" t="inlineStr"/>
-      <c r="L14" s="16" t="inlineStr"/>
-      <c r="M14" s="16" t="inlineStr"/>
-      <c r="N14" s="16" t="inlineStr"/>
-      <c r="O14" s="16" t="inlineStr"/>
-      <c r="P14" s="16" t="inlineStr">
+      <c r="J16" s="17" t="inlineStr"/>
+      <c r="K16" s="17" t="inlineStr"/>
+      <c r="L16" s="17" t="inlineStr"/>
+      <c r="M16" s="17" t="inlineStr"/>
+      <c r="N16" s="17" t="inlineStr"/>
+      <c r="O16" s="17" t="inlineStr"/>
+      <c r="P16" s="17" t="inlineStr">
         <is>
           <t>GitHub Activity Report</t>
         </is>
       </c>
-      <c r="Q14" s="16" t="n">
+      <c r="Q16" s="17" t="n">
         <v>24234243976</v>
       </c>
-      <c r="R14" s="16" t="inlineStr">
+      <c r="R16" s="17" t="inlineStr">
         <is>
           <t>push</t>
         </is>
       </c>
-      <c r="S14" s="16" t="inlineStr">
+      <c r="S16" s="17" t="inlineStr">
         <is>
           <t>2026-04-10T08:35:20Z</t>
         </is>
       </c>
-      <c r="T14" s="16" t="inlineStr">
+      <c r="T16" s="17" t="inlineStr">
         <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="U14" s="17" t="inlineStr">
+      <c r="U16" s="18" t="inlineStr">
         <is>
           <t>success</t>
         </is>
       </c>
-      <c r="V14" s="16" t="inlineStr"/>
-      <c r="W14" s="16" t="inlineStr"/>
-      <c r="X14" s="16" t="inlineStr"/>
-      <c r="Y14" s="16" t="inlineStr"/>
-      <c r="Z14" s="16" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="16" t="inlineStr">
-        <is>
-          <t>git-report</t>
-        </is>
-      </c>
-      <c r="B15" s="16" t="inlineStr">
-        <is>
-          <t>vidyakar-whitedev</t>
-        </is>
-      </c>
-      <c r="C15" s="16" t="inlineStr">
+      <c r="V16" s="17" t="inlineStr"/>
+      <c r="W16" s="17" t="inlineStr"/>
+      <c r="X16" s="17" t="inlineStr"/>
+      <c r="Y16" s="17" t="inlineStr"/>
+      <c r="Z16" s="17" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="17" t="inlineStr">
+        <is>
+          <t>git-report</t>
+        </is>
+      </c>
+      <c r="B17" s="17" t="inlineStr">
+        <is>
+          <t>vidyakar-whitedev</t>
+        </is>
+      </c>
+      <c r="C17" s="17" t="inlineStr">
         <is>
           <t>public</t>
         </is>
       </c>
-      <c r="D15" s="16" t="inlineStr">
+      <c r="D17" s="17" t="inlineStr">
         <is>
           <t>main</t>
         </is>
       </c>
-      <c r="E15" s="16" t="inlineStr">
+      <c r="E17" s="17" t="inlineStr">
         <is>
           <t>9d220c5657c48c13ca17102c507b756edbba9215</t>
         </is>
       </c>
-      <c r="F15" s="16" t="inlineStr">
+      <c r="F17" s="17" t="inlineStr">
         <is>
           <t>test-8</t>
         </is>
       </c>
-      <c r="G15" s="16" t="inlineStr">
+      <c r="G17" s="17" t="inlineStr">
         <is>
           <t>“Vidyakar”</t>
         </is>
       </c>
-      <c r="H15" s="16" t="inlineStr">
+      <c r="H17" s="17" t="inlineStr">
         <is>
           <t>2026-04-10T08:32:22Z</t>
         </is>
       </c>
-      <c r="I15" s="16" t="inlineStr">
+      <c r="I17" s="17" t="inlineStr">
         <is>
           <t>main</t>
         </is>
       </c>
-      <c r="J15" s="16" t="inlineStr"/>
-      <c r="K15" s="16" t="inlineStr"/>
-      <c r="L15" s="16" t="inlineStr"/>
-      <c r="M15" s="16" t="inlineStr"/>
-      <c r="N15" s="16" t="inlineStr"/>
-      <c r="O15" s="16" t="inlineStr"/>
-      <c r="P15" s="16" t="inlineStr">
+      <c r="J17" s="17" t="inlineStr"/>
+      <c r="K17" s="17" t="inlineStr"/>
+      <c r="L17" s="17" t="inlineStr"/>
+      <c r="M17" s="17" t="inlineStr"/>
+      <c r="N17" s="17" t="inlineStr"/>
+      <c r="O17" s="17" t="inlineStr"/>
+      <c r="P17" s="17" t="inlineStr">
         <is>
           <t>GitHub Activity Report</t>
         </is>
       </c>
-      <c r="Q15" s="16" t="n">
+      <c r="Q17" s="17" t="n">
         <v>24234135440</v>
       </c>
-      <c r="R15" s="16" t="inlineStr">
+      <c r="R17" s="17" t="inlineStr">
         <is>
           <t>push</t>
         </is>
       </c>
-      <c r="S15" s="16" t="inlineStr">
+      <c r="S17" s="17" t="inlineStr">
         <is>
           <t>2026-04-10T08:32:30Z</t>
         </is>
       </c>
-      <c r="T15" s="16" t="inlineStr">
+      <c r="T17" s="17" t="inlineStr">
         <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="U15" s="17" t="inlineStr">
+      <c r="U17" s="18" t="inlineStr">
         <is>
           <t>success</t>
         </is>
       </c>
-      <c r="V15" s="16" t="inlineStr"/>
-      <c r="W15" s="16" t="inlineStr"/>
-      <c r="X15" s="16" t="inlineStr"/>
-      <c r="Y15" s="16" t="inlineStr"/>
-      <c r="Z15" s="16" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="16" t="inlineStr">
-        <is>
-          <t>git-report</t>
-        </is>
-      </c>
-      <c r="B16" s="16" t="inlineStr">
-        <is>
-          <t>vidyakar-whitedev</t>
-        </is>
-      </c>
-      <c r="C16" s="16" t="inlineStr">
+      <c r="V17" s="17" t="inlineStr"/>
+      <c r="W17" s="17" t="inlineStr"/>
+      <c r="X17" s="17" t="inlineStr"/>
+      <c r="Y17" s="17" t="inlineStr"/>
+      <c r="Z17" s="17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>git-report</t>
+        </is>
+      </c>
+      <c r="B18" s="17" t="inlineStr">
+        <is>
+          <t>vidyakar-whitedev</t>
+        </is>
+      </c>
+      <c r="C18" s="17" t="inlineStr">
         <is>
           <t>public</t>
         </is>
       </c>
-      <c r="D16" s="16" t="inlineStr">
+      <c r="D18" s="17" t="inlineStr">
         <is>
           <t>main</t>
         </is>
       </c>
-      <c r="E16" s="16" t="inlineStr">
+      <c r="E18" s="17" t="inlineStr">
         <is>
           <t>981fe60621c98393750f79dd815a0ea7e4aed75e</t>
         </is>
       </c>
-      <c r="F16" s="16" t="inlineStr">
+      <c r="F18" s="17" t="inlineStr">
         <is>
           <t>test-8</t>
         </is>
       </c>
-      <c r="G16" s="16" t="inlineStr">
+      <c r="G18" s="17" t="inlineStr">
         <is>
           <t>“Vidyakar”</t>
         </is>
       </c>
-      <c r="H16" s="16" t="inlineStr">
+      <c r="H18" s="17" t="inlineStr">
         <is>
           <t>2026-04-10T08:27:06Z</t>
         </is>
       </c>
-      <c r="I16" s="16" t="inlineStr">
+      <c r="I18" s="17" t="inlineStr">
         <is>
           <t>main</t>
         </is>
       </c>
-      <c r="J16" s="16" t="inlineStr"/>
-      <c r="K16" s="16" t="inlineStr"/>
-      <c r="L16" s="16" t="inlineStr"/>
-      <c r="M16" s="16" t="inlineStr"/>
-      <c r="N16" s="16" t="inlineStr"/>
-      <c r="O16" s="16" t="inlineStr"/>
-      <c r="P16" s="16" t="inlineStr">
+      <c r="J18" s="17" t="inlineStr"/>
+      <c r="K18" s="17" t="inlineStr"/>
+      <c r="L18" s="17" t="inlineStr"/>
+      <c r="M18" s="17" t="inlineStr"/>
+      <c r="N18" s="17" t="inlineStr"/>
+      <c r="O18" s="17" t="inlineStr"/>
+      <c r="P18" s="17" t="inlineStr">
         <is>
           <t>GitHub Activity Report</t>
         </is>
       </c>
-      <c r="Q16" s="16" t="n">
+      <c r="Q18" s="17" t="n">
         <v>24233936358</v>
       </c>
-      <c r="R16" s="16" t="inlineStr">
+      <c r="R18" s="17" t="inlineStr">
         <is>
           <t>push</t>
         </is>
       </c>
-      <c r="S16" s="16" t="inlineStr">
+      <c r="S18" s="17" t="inlineStr">
         <is>
           <t>2026-04-10T08:27:14Z</t>
         </is>
       </c>
-      <c r="T16" s="16" t="inlineStr">
+      <c r="T18" s="17" t="inlineStr">
         <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="U16" s="17" t="inlineStr">
+      <c r="U18" s="18" t="inlineStr">
         <is>
           <t>success</t>
         </is>
       </c>
-      <c r="V16" s="16" t="inlineStr"/>
-      <c r="W16" s="16" t="inlineStr"/>
-      <c r="X16" s="16" t="inlineStr"/>
-      <c r="Y16" s="16" t="inlineStr"/>
-      <c r="Z16" s="16" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="16" t="inlineStr">
-        <is>
-          <t>git-report</t>
-        </is>
-      </c>
-      <c r="B17" s="16" t="inlineStr">
-        <is>
-          <t>vidyakar-whitedev</t>
-        </is>
-      </c>
-      <c r="C17" s="16" t="inlineStr">
+      <c r="V18" s="17" t="inlineStr"/>
+      <c r="W18" s="17" t="inlineStr"/>
+      <c r="X18" s="17" t="inlineStr"/>
+      <c r="Y18" s="17" t="inlineStr"/>
+      <c r="Z18" s="17" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="17" t="inlineStr">
+        <is>
+          <t>git-report</t>
+        </is>
+      </c>
+      <c r="B19" s="17" t="inlineStr">
+        <is>
+          <t>vidyakar-whitedev</t>
+        </is>
+      </c>
+      <c r="C19" s="17" t="inlineStr">
         <is>
           <t>public</t>
         </is>
       </c>
-      <c r="D17" s="16" t="inlineStr">
+      <c r="D19" s="17" t="inlineStr">
         <is>
           <t>main</t>
         </is>
       </c>
-      <c r="E17" s="16" t="inlineStr">
+      <c r="E19" s="17" t="inlineStr">
         <is>
           <t>3cfdf96375ed8ea8c83b95f26b9c87428b8bc8b9</t>
         </is>
       </c>
-      <c r="F17" s="16" t="inlineStr">
+      <c r="F19" s="17" t="inlineStr">
         <is>
           <t>test-1</t>
         </is>
       </c>
-      <c r="G17" s="16" t="inlineStr">
+      <c r="G19" s="17" t="inlineStr">
         <is>
           <t>“Vidyakar”</t>
         </is>
       </c>
-      <c r="H17" s="16" t="inlineStr">
+      <c r="H19" s="17" t="inlineStr">
         <is>
           <t>2026-04-10T08:18:15Z</t>
         </is>
       </c>
-      <c r="I17" s="16" t="inlineStr">
+      <c r="I19" s="17" t="inlineStr">
         <is>
           <t>main</t>
         </is>
       </c>
-      <c r="J17" s="16" t="inlineStr"/>
-      <c r="K17" s="16" t="inlineStr"/>
-      <c r="L17" s="16" t="inlineStr"/>
-      <c r="M17" s="16" t="inlineStr"/>
-      <c r="N17" s="16" t="inlineStr"/>
-      <c r="O17" s="16" t="inlineStr"/>
-      <c r="P17" s="16" t="inlineStr">
+      <c r="J19" s="17" t="inlineStr"/>
+      <c r="K19" s="17" t="inlineStr"/>
+      <c r="L19" s="17" t="inlineStr"/>
+      <c r="M19" s="17" t="inlineStr"/>
+      <c r="N19" s="17" t="inlineStr"/>
+      <c r="O19" s="17" t="inlineStr"/>
+      <c r="P19" s="17" t="inlineStr">
         <is>
           <t>GitHub Activity Report</t>
         </is>
       </c>
-      <c r="Q17" s="16" t="n">
+      <c r="Q19" s="17" t="n">
         <v>24233616319</v>
       </c>
-      <c r="R17" s="16" t="inlineStr">
+      <c r="R19" s="17" t="inlineStr">
         <is>
           <t>push</t>
         </is>
       </c>
-      <c r="S17" s="16" t="inlineStr">
+      <c r="S19" s="17" t="inlineStr">
         <is>
           <t>2026-04-10T08:18:28Z</t>
         </is>
       </c>
-      <c r="T17" s="16" t="inlineStr">
+      <c r="T19" s="17" t="inlineStr">
         <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="U17" s="17" t="inlineStr">
+      <c r="U19" s="18" t="inlineStr">
         <is>
           <t>success</t>
         </is>
       </c>
-      <c r="V17" s="16" t="inlineStr"/>
-      <c r="W17" s="16" t="inlineStr"/>
-      <c r="X17" s="16" t="inlineStr"/>
-      <c r="Y17" s="16" t="inlineStr"/>
-      <c r="Z17" s="16" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="16" t="inlineStr">
-        <is>
-          <t>git-report</t>
-        </is>
-      </c>
-      <c r="B18" s="16" t="inlineStr">
-        <is>
-          <t>vidyakar-whitedev</t>
-        </is>
-      </c>
-      <c r="C18" s="16" t="inlineStr">
+      <c r="V19" s="17" t="inlineStr"/>
+      <c r="W19" s="17" t="inlineStr"/>
+      <c r="X19" s="17" t="inlineStr"/>
+      <c r="Y19" s="17" t="inlineStr"/>
+      <c r="Z19" s="17" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>git-report</t>
+        </is>
+      </c>
+      <c r="B20" s="17" t="inlineStr">
+        <is>
+          <t>vidyakar-whitedev</t>
+        </is>
+      </c>
+      <c r="C20" s="17" t="inlineStr">
         <is>
           <t>public</t>
         </is>
       </c>
-      <c r="D18" s="16" t="inlineStr">
+      <c r="D20" s="17" t="inlineStr">
         <is>
           <t>main</t>
         </is>
       </c>
-      <c r="E18" s="16" t="inlineStr">
+      <c r="E20" s="17" t="inlineStr">
         <is>
           <t>ad211e0513d37204ee54168120dec41978cc6fb4</t>
         </is>
       </c>
-      <c r="F18" s="16" t="inlineStr">
+      <c r="F20" s="17" t="inlineStr">
         <is>
           <t>new code change</t>
         </is>
       </c>
-      <c r="G18" s="16" t="inlineStr">
+      <c r="G20" s="17" t="inlineStr">
         <is>
           <t>“Vidyakar”</t>
         </is>
       </c>
-      <c r="H18" s="16" t="inlineStr">
+      <c r="H20" s="17" t="inlineStr">
         <is>
           <t>2026-04-06T15:32:05Z</t>
         </is>
       </c>
-      <c r="I18" s="16" t="inlineStr">
+      <c r="I20" s="17" t="inlineStr">
         <is>
           <t>main</t>
         </is>
       </c>
-      <c r="J18" s="16" t="inlineStr"/>
-      <c r="K18" s="16" t="inlineStr"/>
-      <c r="L18" s="16" t="inlineStr"/>
-      <c r="M18" s="16" t="inlineStr"/>
-      <c r="N18" s="16" t="inlineStr"/>
-      <c r="O18" s="16" t="inlineStr"/>
-      <c r="P18" s="16" t="inlineStr">
+      <c r="J20" s="17" t="inlineStr"/>
+      <c r="K20" s="17" t="inlineStr"/>
+      <c r="L20" s="17" t="inlineStr"/>
+      <c r="M20" s="17" t="inlineStr"/>
+      <c r="N20" s="17" t="inlineStr"/>
+      <c r="O20" s="17" t="inlineStr"/>
+      <c r="P20" s="17" t="inlineStr">
         <is>
           <t>GitHub Activity Report</t>
         </is>
       </c>
-      <c r="Q18" s="16" t="n">
+      <c r="Q20" s="17" t="n">
         <v>24038137070</v>
       </c>
-      <c r="R18" s="16" t="inlineStr">
+      <c r="R20" s="17" t="inlineStr">
         <is>
           <t>push</t>
         </is>
       </c>
-      <c r="S18" s="16" t="inlineStr">
+      <c r="S20" s="17" t="inlineStr">
         <is>
           <t>2026-04-06T15:32:18Z</t>
         </is>
       </c>
-      <c r="T18" s="16" t="inlineStr">
+      <c r="T20" s="17" t="inlineStr">
         <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="U18" s="17" t="inlineStr">
+      <c r="U20" s="18" t="inlineStr">
         <is>
           <t>success</t>
         </is>
       </c>
-      <c r="V18" s="16" t="inlineStr"/>
-      <c r="W18" s="16" t="inlineStr"/>
-      <c r="X18" s="16" t="inlineStr"/>
-      <c r="Y18" s="16" t="inlineStr"/>
-      <c r="Z18" s="16" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="16" t="inlineStr">
-        <is>
-          <t>git-report</t>
-        </is>
-      </c>
-      <c r="B19" s="16" t="inlineStr">
-        <is>
-          <t>vidyakar-whitedev</t>
-        </is>
-      </c>
-      <c r="C19" s="16" t="inlineStr">
+      <c r="V20" s="17" t="inlineStr"/>
+      <c r="W20" s="17" t="inlineStr"/>
+      <c r="X20" s="17" t="inlineStr"/>
+      <c r="Y20" s="17" t="inlineStr"/>
+      <c r="Z20" s="17" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="17" t="inlineStr">
+        <is>
+          <t>git-report</t>
+        </is>
+      </c>
+      <c r="B21" s="17" t="inlineStr">
+        <is>
+          <t>vidyakar-whitedev</t>
+        </is>
+      </c>
+      <c r="C21" s="17" t="inlineStr">
         <is>
           <t>public</t>
         </is>
       </c>
-      <c r="D19" s="16" t="inlineStr">
+      <c r="D21" s="17" t="inlineStr">
         <is>
           <t>main</t>
         </is>
       </c>
-      <c r="E19" s="16" t="inlineStr">
+      <c r="E21" s="17" t="inlineStr">
         <is>
           <t>21f8e2bcc8765be2c9dd97d0d839686b7afe3de1</t>
         </is>
       </c>
-      <c r="F19" s="16" t="inlineStr">
+      <c r="F21" s="17" t="inlineStr">
         <is>
           <t>new code change</t>
         </is>
       </c>
-      <c r="G19" s="16" t="inlineStr">
+      <c r="G21" s="17" t="inlineStr">
         <is>
           <t>“Vidyakar”</t>
         </is>
       </c>
-      <c r="H19" s="16" t="inlineStr">
+      <c r="H21" s="17" t="inlineStr">
         <is>
           <t>2026-04-06T12:24:00Z</t>
         </is>
       </c>
-      <c r="I19" s="16" t="inlineStr">
+      <c r="I21" s="17" t="inlineStr">
         <is>
           <t>git-report-poc2</t>
         </is>
       </c>
-      <c r="J19" s="16" t="inlineStr"/>
-      <c r="K19" s="16" t="inlineStr"/>
-      <c r="L19" s="16" t="inlineStr"/>
-      <c r="M19" s="16" t="inlineStr"/>
-      <c r="N19" s="16" t="inlineStr"/>
-      <c r="O19" s="16" t="inlineStr"/>
-      <c r="P19" s="16" t="inlineStr">
+      <c r="J21" s="17" t="inlineStr"/>
+      <c r="K21" s="17" t="inlineStr"/>
+      <c r="L21" s="17" t="inlineStr"/>
+      <c r="M21" s="17" t="inlineStr"/>
+      <c r="N21" s="17" t="inlineStr"/>
+      <c r="O21" s="17" t="inlineStr"/>
+      <c r="P21" s="17" t="inlineStr">
         <is>
           <t>GitHub Activity Report</t>
         </is>
       </c>
-      <c r="Q19" s="16" t="n">
+      <c r="Q21" s="17" t="n">
         <v>24031673216</v>
       </c>
-      <c r="R19" s="16" t="inlineStr">
+      <c r="R21" s="17" t="inlineStr">
         <is>
           <t>push</t>
         </is>
       </c>
-      <c r="S19" s="16" t="inlineStr">
+      <c r="S21" s="17" t="inlineStr">
         <is>
           <t>2026-04-06T12:24:13Z</t>
         </is>
       </c>
-      <c r="T19" s="16" t="inlineStr">
+      <c r="T21" s="17" t="inlineStr">
         <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="U19" s="17" t="inlineStr">
+      <c r="U21" s="18" t="inlineStr">
         <is>
           <t>success</t>
         </is>
       </c>
-      <c r="V19" s="16" t="inlineStr"/>
-      <c r="W19" s="16" t="inlineStr"/>
-      <c r="X19" s="16" t="inlineStr"/>
-      <c r="Y19" s="16" t="inlineStr"/>
-      <c r="Z19" s="16" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="19" t="inlineStr">
-        <is>
-          <t>git-report</t>
-        </is>
-      </c>
-      <c r="B20" s="19" t="inlineStr">
-        <is>
-          <t>vidyakar-whitedev</t>
-        </is>
-      </c>
-      <c r="C20" s="19" t="inlineStr">
-        <is>
-          <t>public</t>
-        </is>
-      </c>
-      <c r="D20" s="19" t="inlineStr">
-        <is>
-          <t>main</t>
-        </is>
-      </c>
-      <c r="E20" s="19" t="inlineStr">
-        <is>
-          <t>5b2c09128fdfda0f63e1f6188832caa277f2af4b</t>
-        </is>
-      </c>
-      <c r="F20" s="19" t="inlineStr">
-        <is>
-          <t>code changed1</t>
-        </is>
-      </c>
-      <c r="G20" s="19" t="inlineStr">
-        <is>
-          <t>“Vidyakar”</t>
-        </is>
-      </c>
-      <c r="H20" s="19" t="inlineStr">
-        <is>
-          <t>2026-04-06T11:54:44Z</t>
-        </is>
-      </c>
-      <c r="I20" s="19" t="inlineStr">
-        <is>
-          <t>git-report-poc2</t>
-        </is>
-      </c>
-      <c r="J20" s="19" t="inlineStr"/>
-      <c r="K20" s="19" t="inlineStr"/>
-      <c r="L20" s="19" t="inlineStr"/>
-      <c r="M20" s="19" t="inlineStr"/>
-      <c r="N20" s="19" t="inlineStr"/>
-      <c r="O20" s="19" t="inlineStr"/>
-      <c r="P20" s="19" t="inlineStr">
-        <is>
-          <t>GitHub Workflow Report</t>
-        </is>
-      </c>
-      <c r="Q20" s="19" t="n">
-        <v>24030846379</v>
-      </c>
-      <c r="R20" s="19" t="inlineStr">
-        <is>
-          <t>workflow_dispatch</t>
-        </is>
-      </c>
-      <c r="S20" s="19" t="inlineStr">
-        <is>
-          <t>2026-04-06T11:55:45Z</t>
-        </is>
-      </c>
-      <c r="T20" s="19" t="inlineStr">
-        <is>
-          <t>completed</t>
-        </is>
-      </c>
-      <c r="U20" s="20" t="inlineStr">
-        <is>
-          <t>failure</t>
-        </is>
-      </c>
-      <c r="V20" s="19" t="inlineStr">
-        <is>
-          <t>Job 'generate_report' step 'Run GitHub Activity Report' failed — 2026-04-06T11:56:06.4378556Z Traceback (most recent call last):</t>
-        </is>
-      </c>
-      <c r="W20" s="19" t="inlineStr">
-        <is>
-          <t>generate_report</t>
-        </is>
-      </c>
-      <c r="X20" s="19" t="inlineStr">
-        <is>
-          <t>Run GitHub Activity Report</t>
-        </is>
-      </c>
-      <c r="Y20" s="19" t="inlineStr">
-        <is>
-          <t>Line 56</t>
-        </is>
-      </c>
-      <c r="Z20" s="19" t="inlineStr">
-        <is>
-          <t>Review the full workflow log in GitHub Actions for the specific error message.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="19" t="inlineStr">
-        <is>
-          <t>git-report</t>
-        </is>
-      </c>
-      <c r="B21" s="19" t="inlineStr">
-        <is>
-          <t>vidyakar-whitedev</t>
-        </is>
-      </c>
-      <c r="C21" s="19" t="inlineStr">
-        <is>
-          <t>public</t>
-        </is>
-      </c>
-      <c r="D21" s="19" t="inlineStr">
-        <is>
-          <t>main</t>
-        </is>
-      </c>
-      <c r="E21" s="19" t="inlineStr">
-        <is>
-          <t>5b2c09128fdfda0f63e1f6188832caa277f2af4b</t>
-        </is>
-      </c>
-      <c r="F21" s="19" t="inlineStr">
-        <is>
-          <t>code changed1</t>
-        </is>
-      </c>
-      <c r="G21" s="19" t="inlineStr">
-        <is>
-          <t>“Vidyakar”</t>
-        </is>
-      </c>
-      <c r="H21" s="19" t="inlineStr">
-        <is>
-          <t>2026-04-06T11:54:44Z</t>
-        </is>
-      </c>
-      <c r="I21" s="19" t="inlineStr">
-        <is>
-          <t>git-report-poc2</t>
-        </is>
-      </c>
-      <c r="J21" s="19" t="inlineStr"/>
-      <c r="K21" s="19" t="inlineStr"/>
-      <c r="L21" s="19" t="inlineStr"/>
-      <c r="M21" s="19" t="inlineStr"/>
-      <c r="N21" s="19" t="inlineStr"/>
-      <c r="O21" s="19" t="inlineStr"/>
-      <c r="P21" s="19" t="inlineStr">
-        <is>
-          <t>GitHub Workflow Report</t>
-        </is>
-      </c>
-      <c r="Q21" s="19" t="n">
-        <v>24030820444</v>
-      </c>
-      <c r="R21" s="19" t="inlineStr">
-        <is>
-          <t>push</t>
-        </is>
-      </c>
-      <c r="S21" s="19" t="inlineStr">
-        <is>
-          <t>2026-04-06T11:54:51Z</t>
-        </is>
-      </c>
-      <c r="T21" s="19" t="inlineStr">
-        <is>
-          <t>completed</t>
-        </is>
-      </c>
-      <c r="U21" s="20" t="inlineStr">
-        <is>
-          <t>failure</t>
-        </is>
-      </c>
-      <c r="V21" s="19" t="inlineStr">
-        <is>
-          <t>Job 'generate_report' step 'Run GitHub Activity Report' failed — 2026-04-06T11:55:12.8179279Z Traceback (most recent call last):</t>
-        </is>
-      </c>
-      <c r="W21" s="19" t="inlineStr">
-        <is>
-          <t>generate_report</t>
-        </is>
-      </c>
-      <c r="X21" s="19" t="inlineStr">
-        <is>
-          <t>Run GitHub Activity Report</t>
-        </is>
-      </c>
-      <c r="Y21" s="19" t="inlineStr">
-        <is>
-          <t>Line 55</t>
-        </is>
-      </c>
-      <c r="Z21" s="19" t="inlineStr">
-        <is>
-          <t>Review the full workflow log in GitHub Actions for the specific error message.</t>
-        </is>
-      </c>
+      <c r="V21" s="17" t="inlineStr"/>
+      <c r="W21" s="17" t="inlineStr"/>
+      <c r="X21" s="17" t="inlineStr"/>
+      <c r="Y21" s="17" t="inlineStr"/>
+      <c r="Z21" s="17" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="19" t="inlineStr">
@@ -2665,12 +2603,12 @@
       </c>
       <c r="E22" s="19" t="inlineStr">
         <is>
-          <t>733b89967b9b4731953302840f2ddb2c20bedf56</t>
+          <t>5b2c09128fdfda0f63e1f6188832caa277f2af4b</t>
         </is>
       </c>
       <c r="F22" s="19" t="inlineStr">
         <is>
-          <t>code changed</t>
+          <t>code changed1</t>
         </is>
       </c>
       <c r="G22" s="19" t="inlineStr">
@@ -2680,7 +2618,7 @@
       </c>
       <c r="H22" s="19" t="inlineStr">
         <is>
-          <t>2026-04-06T10:52:40Z</t>
+          <t>2026-04-06T11:54:44Z</t>
         </is>
       </c>
       <c r="I22" s="19" t="inlineStr">
@@ -2700,16 +2638,16 @@
         </is>
       </c>
       <c r="Q22" s="19" t="n">
-        <v>24029078530</v>
+        <v>24030846379</v>
       </c>
       <c r="R22" s="19" t="inlineStr">
         <is>
-          <t>push</t>
+          <t>workflow_dispatch</t>
         </is>
       </c>
       <c r="S22" s="19" t="inlineStr">
         <is>
-          <t>2026-04-06T10:52:49Z</t>
+          <t>2026-04-06T11:55:45Z</t>
         </is>
       </c>
       <c r="T22" s="19" t="inlineStr">
@@ -2724,7 +2662,7 @@
       </c>
       <c r="V22" s="19" t="inlineStr">
         <is>
-          <t>Job 'generate_report' step 'Set up job' failed — 2026-04-06T10:52:53.8436108Z ##[error]This request has been automatically failed because it uses a deprecated version of</t>
+          <t>Job 'generate_report' step 'Run GitHub Activity Report' failed — 2026-04-06T11:56:06.4378556Z Traceback (most recent call last):</t>
         </is>
       </c>
       <c r="W22" s="19" t="inlineStr">
@@ -2734,12 +2672,12 @@
       </c>
       <c r="X22" s="19" t="inlineStr">
         <is>
-          <t>Set up job</t>
+          <t>Run GitHub Activity Report</t>
         </is>
       </c>
       <c r="Y22" s="19" t="inlineStr">
         <is>
-          <t>Line 52</t>
+          <t>Line 56</t>
         </is>
       </c>
       <c r="Z22" s="19" t="inlineStr">
@@ -2771,12 +2709,12 @@
       </c>
       <c r="E23" s="19" t="inlineStr">
         <is>
-          <t>aedf77ebc8e0433ebbe37ca97908ee5caf3929d6</t>
+          <t>5b2c09128fdfda0f63e1f6188832caa277f2af4b</t>
         </is>
       </c>
       <c r="F23" s="19" t="inlineStr">
         <is>
-          <t>code changd</t>
+          <t>code changed1</t>
         </is>
       </c>
       <c r="G23" s="19" t="inlineStr">
@@ -2786,7 +2724,7 @@
       </c>
       <c r="H23" s="19" t="inlineStr">
         <is>
-          <t>2026-04-06T10:44:38Z</t>
+          <t>2026-04-06T11:54:44Z</t>
         </is>
       </c>
       <c r="I23" s="19" t="inlineStr">
@@ -2806,7 +2744,7 @@
         </is>
       </c>
       <c r="Q23" s="19" t="n">
-        <v>24028853853</v>
+        <v>24030820444</v>
       </c>
       <c r="R23" s="19" t="inlineStr">
         <is>
@@ -2815,7 +2753,7 @@
       </c>
       <c r="S23" s="19" t="inlineStr">
         <is>
-          <t>2026-04-06T10:44:47Z</t>
+          <t>2026-04-06T11:54:51Z</t>
         </is>
       </c>
       <c r="T23" s="19" t="inlineStr">
@@ -2830,27 +2768,27 @@
       </c>
       <c r="V23" s="19" t="inlineStr">
         <is>
-          <t>Job 'report' step 'Run GitHub Workflow Report' failed — 2026-04-06T10:45:06.2894428Z ERROR: No repositories found. Check GH_ORG value and token permissions.</t>
+          <t>Job 'generate_report' step 'Run GitHub Activity Report' failed — 2026-04-06T11:55:12.8179279Z Traceback (most recent call last):</t>
         </is>
       </c>
       <c r="W23" s="19" t="inlineStr">
         <is>
-          <t>report</t>
+          <t>generate_report</t>
         </is>
       </c>
       <c r="X23" s="19" t="inlineStr">
         <is>
-          <t>Run GitHub Workflow Report</t>
+          <t>Run GitHub Activity Report</t>
         </is>
       </c>
       <c r="Y23" s="19" t="inlineStr">
         <is>
-          <t>Line 45</t>
+          <t>Line 55</t>
         </is>
       </c>
       <c r="Z23" s="19" t="inlineStr">
         <is>
-          <t>Auth/permission error — verify GH_PAT scopes and that repository secrets are correctly configured.</t>
+          <t>Review the full workflow log in GitHub Actions for the specific error message.</t>
         </is>
       </c>
     </row>
@@ -2877,22 +2815,22 @@
       </c>
       <c r="E24" s="19" t="inlineStr">
         <is>
-          <t>5feb9eb868fd9ff9e4a7150d13cb3252d843c106</t>
+          <t>733b89967b9b4731953302840f2ddb2c20bedf56</t>
         </is>
       </c>
       <c r="F24" s="19" t="inlineStr">
         <is>
-          <t>Update demo.txt</t>
+          <t>code changed</t>
         </is>
       </c>
       <c r="G24" s="19" t="inlineStr">
         <is>
-          <t>vidyakar-whitedev</t>
+          <t>“Vidyakar”</t>
         </is>
       </c>
       <c r="H24" s="19" t="inlineStr">
         <is>
-          <t>2026-04-06T10:31:56Z</t>
+          <t>2026-04-06T10:52:40Z</t>
         </is>
       </c>
       <c r="I24" s="19" t="inlineStr">
@@ -2912,7 +2850,7 @@
         </is>
       </c>
       <c r="Q24" s="19" t="n">
-        <v>24028486557</v>
+        <v>24029078530</v>
       </c>
       <c r="R24" s="19" t="inlineStr">
         <is>
@@ -2921,7 +2859,7 @@
       </c>
       <c r="S24" s="19" t="inlineStr">
         <is>
-          <t>2026-04-06T10:39:17Z</t>
+          <t>2026-04-06T10:52:49Z</t>
         </is>
       </c>
       <c r="T24" s="19" t="inlineStr">
@@ -2936,22 +2874,22 @@
       </c>
       <c r="V24" s="19" t="inlineStr">
         <is>
-          <t>Job 'report' step 'Run GitHub Workflow Report' failed — 2026-04-06T10:39:35.5521802Z Traceback (most recent call last):</t>
+          <t>Job 'generate_report' step 'Set up job' failed — 2026-04-06T10:52:53.8436108Z ##[error]This request has been automatically failed because it uses a deprecated version of</t>
         </is>
       </c>
       <c r="W24" s="19" t="inlineStr">
         <is>
-          <t>report</t>
+          <t>generate_report</t>
         </is>
       </c>
       <c r="X24" s="19" t="inlineStr">
         <is>
-          <t>Run GitHub Workflow Report</t>
+          <t>Set up job</t>
         </is>
       </c>
       <c r="Y24" s="19" t="inlineStr">
         <is>
-          <t>Line 39</t>
+          <t>Line 52</t>
         </is>
       </c>
       <c r="Z24" s="19" t="inlineStr">
@@ -2983,12 +2921,12 @@
       </c>
       <c r="E25" s="19" t="inlineStr">
         <is>
-          <t>2fcbd831207ea4821a39ee88d33aa21454ca19e3</t>
+          <t>aedf77ebc8e0433ebbe37ca97908ee5caf3929d6</t>
         </is>
       </c>
       <c r="F25" s="19" t="inlineStr">
         <is>
-          <t>code changed@v1</t>
+          <t>code changd</t>
         </is>
       </c>
       <c r="G25" s="19" t="inlineStr">
@@ -2998,7 +2936,7 @@
       </c>
       <c r="H25" s="19" t="inlineStr">
         <is>
-          <t>2026-04-06T10:28:57Z</t>
+          <t>2026-04-06T10:44:38Z</t>
         </is>
       </c>
       <c r="I25" s="19" t="inlineStr">
@@ -3018,7 +2956,7 @@
         </is>
       </c>
       <c r="Q25" s="19" t="n">
-        <v>24028398959</v>
+        <v>24028853853</v>
       </c>
       <c r="R25" s="19" t="inlineStr">
         <is>
@@ -3027,7 +2965,7 @@
       </c>
       <c r="S25" s="19" t="inlineStr">
         <is>
-          <t>2026-04-06T10:29:06Z</t>
+          <t>2026-04-06T10:44:47Z</t>
         </is>
       </c>
       <c r="T25" s="19" t="inlineStr">
@@ -3042,7 +2980,7 @@
       </c>
       <c r="V25" s="19" t="inlineStr">
         <is>
-          <t>Job 'report' step 'Run GitHub Workflow Report' failed — 2026-04-06T10:29:24.4401300Z Traceback (most recent call last):</t>
+          <t>Job 'report' step 'Run GitHub Workflow Report' failed — 2026-04-06T10:45:06.2894428Z ERROR: No repositories found. Check GH_ORG value and token permissions.</t>
         </is>
       </c>
       <c r="W25" s="19" t="inlineStr">
@@ -3057,7 +2995,7 @@
       </c>
       <c r="Y25" s="19" t="inlineStr">
         <is>
-          <t>Line 29</t>
+          <t>Line 45</t>
         </is>
       </c>
       <c r="Z25" s="19" t="inlineStr">
@@ -3089,22 +3027,22 @@
       </c>
       <c r="E26" s="19" t="inlineStr">
         <is>
-          <t>37ddfe095b13b5e65a98ff2072c4bbb77cde7c1b</t>
+          <t>5feb9eb868fd9ff9e4a7150d13cb3252d843c106</t>
         </is>
       </c>
       <c r="F26" s="19" t="inlineStr">
         <is>
-          <t>code changed</t>
+          <t>Update demo.txt</t>
         </is>
       </c>
       <c r="G26" s="19" t="inlineStr">
         <is>
-          <t>“Vidyakar”</t>
+          <t>vidyakar-whitedev</t>
         </is>
       </c>
       <c r="H26" s="19" t="inlineStr">
         <is>
-          <t>2026-04-06T10:22:31Z</t>
+          <t>2026-04-06T10:31:56Z</t>
         </is>
       </c>
       <c r="I26" s="19" t="inlineStr">
@@ -3124,7 +3062,7 @@
         </is>
       </c>
       <c r="Q26" s="19" t="n">
-        <v>24028208740</v>
+        <v>24028486557</v>
       </c>
       <c r="R26" s="19" t="inlineStr">
         <is>
@@ -3133,7 +3071,7 @@
       </c>
       <c r="S26" s="19" t="inlineStr">
         <is>
-          <t>2026-04-06T10:22:38Z</t>
+          <t>2026-04-06T10:39:17Z</t>
         </is>
       </c>
       <c r="T26" s="19" t="inlineStr">
@@ -3148,7 +3086,7 @@
       </c>
       <c r="V26" s="19" t="inlineStr">
         <is>
-          <t>Job 'report' step 'Install dependencies' failed — 2026-04-06T10:22:44.0853785Z ERROR: Could not open requirements file: [Errno 2] No such file or directory: 'requirements</t>
+          <t>Job 'report' step 'Run GitHub Workflow Report' failed — 2026-04-06T10:39:35.5521802Z Traceback (most recent call last):</t>
         </is>
       </c>
       <c r="W26" s="19" t="inlineStr">
@@ -3158,17 +3096,17 @@
       </c>
       <c r="X26" s="19" t="inlineStr">
         <is>
-          <t>Install dependencies</t>
+          <t>Run GitHub Workflow Report</t>
         </is>
       </c>
       <c r="Y26" s="19" t="inlineStr">
         <is>
-          <t>Line 22</t>
+          <t>Line 39</t>
         </is>
       </c>
       <c r="Z26" s="19" t="inlineStr">
         <is>
-          <t>Dependency error — run `pip install -r requirements.txt` or `npm install` and verify package versions.</t>
+          <t>Review the full workflow log in GitHub Actions for the specific error message.</t>
         </is>
       </c>
     </row>
@@ -3195,12 +3133,12 @@
       </c>
       <c r="E27" s="19" t="inlineStr">
         <is>
-          <t>74dcfb5e2119b07af9671cc4c8396585d44a6fb8</t>
+          <t>2fcbd831207ea4821a39ee88d33aa21454ca19e3</t>
         </is>
       </c>
       <c r="F27" s="19" t="inlineStr">
         <is>
-          <t>code</t>
+          <t>code changed@v1</t>
         </is>
       </c>
       <c r="G27" s="19" t="inlineStr">
@@ -3210,7 +3148,7 @@
       </c>
       <c r="H27" s="19" t="inlineStr">
         <is>
-          <t>2026-04-06T10:21:05Z</t>
+          <t>2026-04-06T10:28:57Z</t>
         </is>
       </c>
       <c r="I27" s="19" t="inlineStr">
@@ -3230,7 +3168,7 @@
         </is>
       </c>
       <c r="Q27" s="19" t="n">
-        <v>24028171694</v>
+        <v>24028398959</v>
       </c>
       <c r="R27" s="19" t="inlineStr">
         <is>
@@ -3239,7 +3177,7 @@
       </c>
       <c r="S27" s="19" t="inlineStr">
         <is>
-          <t>2026-04-06T10:21:19Z</t>
+          <t>2026-04-06T10:29:06Z</t>
         </is>
       </c>
       <c r="T27" s="19" t="inlineStr">
@@ -3254,7 +3192,7 @@
       </c>
       <c r="V27" s="19" t="inlineStr">
         <is>
-          <t>Job 'report' step 'Install dependencies' failed — 2026-04-06T10:21:26.0154829Z ERROR: Could not open requirements file: [Errno 2] No such file or directory: 'requirements</t>
+          <t>Job 'report' step 'Run GitHub Workflow Report' failed — 2026-04-06T10:29:24.4401300Z Traceback (most recent call last):</t>
         </is>
       </c>
       <c r="W27" s="19" t="inlineStr">
@@ -3264,17 +3202,17 @@
       </c>
       <c r="X27" s="19" t="inlineStr">
         <is>
-          <t>Install dependencies</t>
+          <t>Run GitHub Workflow Report</t>
         </is>
       </c>
       <c r="Y27" s="19" t="inlineStr">
         <is>
-          <t>Line 21</t>
+          <t>Line 29</t>
         </is>
       </c>
       <c r="Z27" s="19" t="inlineStr">
         <is>
-          <t>Dependency error — run `pip install -r requirements.txt` or `npm install` and verify package versions.</t>
+          <t>Auth/permission error — verify GH_PAT scopes and that repository secrets are correctly configured.</t>
         </is>
       </c>
     </row>
@@ -3301,22 +3239,22 @@
       </c>
       <c r="E28" s="19" t="inlineStr">
         <is>
-          <t>5ff73a4b92ec974d47dc4998318d0eb25003ef50</t>
+          <t>37ddfe095b13b5e65a98ff2072c4bbb77cde7c1b</t>
         </is>
       </c>
       <c r="F28" s="19" t="inlineStr">
         <is>
-          <t>Enhance workflow with caching and Node.js versioning</t>
+          <t>code changed</t>
         </is>
       </c>
       <c r="G28" s="19" t="inlineStr">
         <is>
-          <t>vidyakar-whitedev</t>
+          <t>“Vidyakar”</t>
         </is>
       </c>
       <c r="H28" s="19" t="inlineStr">
         <is>
-          <t>2026-04-06T10:08:38Z</t>
+          <t>2026-04-06T10:22:31Z</t>
         </is>
       </c>
       <c r="I28" s="19" t="inlineStr">
@@ -3336,7 +3274,7 @@
         </is>
       </c>
       <c r="Q28" s="19" t="n">
-        <v>24027807973</v>
+        <v>24028208740</v>
       </c>
       <c r="R28" s="19" t="inlineStr">
         <is>
@@ -3345,7 +3283,7 @@
       </c>
       <c r="S28" s="19" t="inlineStr">
         <is>
-          <t>2026-04-06T10:08:40Z</t>
+          <t>2026-04-06T10:22:38Z</t>
         </is>
       </c>
       <c r="T28" s="19" t="inlineStr">
@@ -3360,7 +3298,7 @@
       </c>
       <c r="V28" s="19" t="inlineStr">
         <is>
-          <t>Job 'report' step 'Install dependencies' failed — 2026-04-06T10:08:48.9456340Z ERROR: Could not open requirements file: [Errno 2] No such file or directory: 'requirements</t>
+          <t>Job 'report' step 'Install dependencies' failed — 2026-04-06T10:22:44.0853785Z ERROR: Could not open requirements file: [Errno 2] No such file or directory: 'requirements</t>
         </is>
       </c>
       <c r="W28" s="19" t="inlineStr">
@@ -3375,7 +3313,7 @@
       </c>
       <c r="Y28" s="19" t="inlineStr">
         <is>
-          <t>Line 08</t>
+          <t>Line 22</t>
         </is>
       </c>
       <c r="Z28" s="19" t="inlineStr">
@@ -3407,22 +3345,22 @@
       </c>
       <c r="E29" s="19" t="inlineStr">
         <is>
-          <t>ad002901ed69655717989c4485c2df1f343c5b15</t>
+          <t>74dcfb5e2119b07af9671cc4c8396585d44a6fb8</t>
         </is>
       </c>
       <c r="F29" s="19" t="inlineStr">
         <is>
-          <t>Fix typo in demo.txt</t>
+          <t>code</t>
         </is>
       </c>
       <c r="G29" s="19" t="inlineStr">
         <is>
-          <t>vidyakar-whitedev</t>
+          <t>“Vidyakar”</t>
         </is>
       </c>
       <c r="H29" s="19" t="inlineStr">
         <is>
-          <t>2026-04-06T10:06:00Z</t>
+          <t>2026-04-06T10:21:05Z</t>
         </is>
       </c>
       <c r="I29" s="19" t="inlineStr">
@@ -3442,7 +3380,7 @@
         </is>
       </c>
       <c r="Q29" s="19" t="n">
-        <v>24027735534</v>
+        <v>24028171694</v>
       </c>
       <c r="R29" s="19" t="inlineStr">
         <is>
@@ -3451,7 +3389,7 @@
       </c>
       <c r="S29" s="19" t="inlineStr">
         <is>
-          <t>2026-04-06T10:06:01Z</t>
+          <t>2026-04-06T10:21:19Z</t>
         </is>
       </c>
       <c r="T29" s="19" t="inlineStr">
@@ -3466,7 +3404,7 @@
       </c>
       <c r="V29" s="19" t="inlineStr">
         <is>
-          <t>Job 'report' step 'Run GitHub Workflow Report' failed — 2026-04-06T10:06:18.4738139Z Traceback (most recent call last):</t>
+          <t>Job 'report' step 'Install dependencies' failed — 2026-04-06T10:21:26.0154829Z ERROR: Could not open requirements file: [Errno 2] No such file or directory: 'requirements</t>
         </is>
       </c>
       <c r="W29" s="19" t="inlineStr">
@@ -3476,17 +3414,17 @@
       </c>
       <c r="X29" s="19" t="inlineStr">
         <is>
-          <t>Run GitHub Workflow Report</t>
+          <t>Install dependencies</t>
         </is>
       </c>
       <c r="Y29" s="19" t="inlineStr">
         <is>
-          <t>Line 06</t>
+          <t>Line 21</t>
         </is>
       </c>
       <c r="Z29" s="19" t="inlineStr">
         <is>
-          <t>Review the full workflow log in GitHub Actions for the specific error message.</t>
+          <t>Dependency error — run `pip install -r requirements.txt` or `npm install` and verify package versions.</t>
         </is>
       </c>
     </row>
@@ -3513,12 +3451,12 @@
       </c>
       <c r="E30" s="19" t="inlineStr">
         <is>
-          <t>06a295fe67b6991a6ba3430be5f485beedd7805f</t>
+          <t>5ff73a4b92ec974d47dc4998318d0eb25003ef50</t>
         </is>
       </c>
       <c r="F30" s="19" t="inlineStr">
         <is>
-          <t>Update workflow_report.yml</t>
+          <t>Enhance workflow with caching and Node.js versioning</t>
         </is>
       </c>
       <c r="G30" s="19" t="inlineStr">
@@ -3528,7 +3466,7 @@
       </c>
       <c r="H30" s="19" t="inlineStr">
         <is>
-          <t>2026-04-06T10:05:48Z</t>
+          <t>2026-04-06T10:08:38Z</t>
         </is>
       </c>
       <c r="I30" s="19" t="inlineStr">
@@ -3548,7 +3486,7 @@
         </is>
       </c>
       <c r="Q30" s="19" t="n">
-        <v>24027729636</v>
+        <v>24027807973</v>
       </c>
       <c r="R30" s="19" t="inlineStr">
         <is>
@@ -3557,7 +3495,7 @@
       </c>
       <c r="S30" s="19" t="inlineStr">
         <is>
-          <t>2026-04-06T10:05:49Z</t>
+          <t>2026-04-06T10:08:40Z</t>
         </is>
       </c>
       <c r="T30" s="19" t="inlineStr">
@@ -3572,7 +3510,7 @@
       </c>
       <c r="V30" s="19" t="inlineStr">
         <is>
-          <t>Job 'report' step 'Run GitHub Workflow Report' failed — 2026-04-06T10:06:03.7190307Z Traceback (most recent call last):</t>
+          <t>Job 'report' step 'Install dependencies' failed — 2026-04-06T10:08:48.9456340Z ERROR: Could not open requirements file: [Errno 2] No such file or directory: 'requirements</t>
         </is>
       </c>
       <c r="W30" s="19" t="inlineStr">
@@ -3582,17 +3520,17 @@
       </c>
       <c r="X30" s="19" t="inlineStr">
         <is>
-          <t>Run GitHub Workflow Report</t>
+          <t>Install dependencies</t>
         </is>
       </c>
       <c r="Y30" s="19" t="inlineStr">
         <is>
-          <t>Line 06</t>
+          <t>Line 08</t>
         </is>
       </c>
       <c r="Z30" s="19" t="inlineStr">
         <is>
-          <t>Review the full workflow log in GitHub Actions for the specific error message.</t>
+          <t>Dependency error — run `pip install -r requirements.txt` or `npm install` and verify package versions.</t>
         </is>
       </c>
     </row>
@@ -3619,12 +3557,12 @@
       </c>
       <c r="E31" s="19" t="inlineStr">
         <is>
-          <t>372cfe624d49eb38f5e8baab2c748007dc54b018</t>
+          <t>ad002901ed69655717989c4485c2df1f343c5b15</t>
         </is>
       </c>
       <c r="F31" s="19" t="inlineStr">
         <is>
-          <t>Update demo.txt</t>
+          <t>Fix typo in demo.txt</t>
         </is>
       </c>
       <c r="G31" s="19" t="inlineStr">
@@ -3634,7 +3572,7 @@
       </c>
       <c r="H31" s="19" t="inlineStr">
         <is>
-          <t>2026-04-06T10:04:34Z</t>
+          <t>2026-04-06T10:06:00Z</t>
         </is>
       </c>
       <c r="I31" s="19" t="inlineStr">
@@ -3654,7 +3592,7 @@
         </is>
       </c>
       <c r="Q31" s="19" t="n">
-        <v>24027694141</v>
+        <v>24027735534</v>
       </c>
       <c r="R31" s="19" t="inlineStr">
         <is>
@@ -3663,7 +3601,7 @@
       </c>
       <c r="S31" s="19" t="inlineStr">
         <is>
-          <t>2026-04-06T10:04:36Z</t>
+          <t>2026-04-06T10:06:01Z</t>
         </is>
       </c>
       <c r="T31" s="19" t="inlineStr">
@@ -3678,7 +3616,7 @@
       </c>
       <c r="V31" s="19" t="inlineStr">
         <is>
-          <t>Job 'report' step 'Set up job' failed — 2026-04-06T10:04:40.5244711Z ##[error]This request has been automatically failed because it uses a deprecated version of</t>
+          <t>Job 'report' step 'Run GitHub Workflow Report' failed — 2026-04-06T10:06:18.4738139Z Traceback (most recent call last):</t>
         </is>
       </c>
       <c r="W31" s="19" t="inlineStr">
@@ -3688,12 +3626,12 @@
       </c>
       <c r="X31" s="19" t="inlineStr">
         <is>
-          <t>Set up job</t>
+          <t>Run GitHub Workflow Report</t>
         </is>
       </c>
       <c r="Y31" s="19" t="inlineStr">
         <is>
-          <t>Line 04</t>
+          <t>Line 06</t>
         </is>
       </c>
       <c r="Z31" s="19" t="inlineStr">
@@ -3725,7 +3663,7 @@
       </c>
       <c r="E32" s="19" t="inlineStr">
         <is>
-          <t>e7bf9d94f807df2e25e29ad5d30bc78e1b2fbd25</t>
+          <t>06a295fe67b6991a6ba3430be5f485beedd7805f</t>
         </is>
       </c>
       <c r="F32" s="19" t="inlineStr">
@@ -3740,7 +3678,7 @@
       </c>
       <c r="H32" s="19" t="inlineStr">
         <is>
-          <t>2026-04-06T10:04:22Z</t>
+          <t>2026-04-06T10:05:48Z</t>
         </is>
       </c>
       <c r="I32" s="19" t="inlineStr">
@@ -3760,7 +3698,7 @@
         </is>
       </c>
       <c r="Q32" s="19" t="n">
-        <v>24027689526</v>
+        <v>24027729636</v>
       </c>
       <c r="R32" s="19" t="inlineStr">
         <is>
@@ -3769,7 +3707,7 @@
       </c>
       <c r="S32" s="19" t="inlineStr">
         <is>
-          <t>2026-04-06T10:04:27Z</t>
+          <t>2026-04-06T10:05:49Z</t>
         </is>
       </c>
       <c r="T32" s="19" t="inlineStr">
@@ -3784,7 +3722,7 @@
       </c>
       <c r="V32" s="19" t="inlineStr">
         <is>
-          <t>Job 'report' step 'Set up job' failed — 2026-04-06T10:04:31.3428173Z ##[error]This request has been automatically failed because it uses a deprecated version of</t>
+          <t>Job 'report' step 'Run GitHub Workflow Report' failed — 2026-04-06T10:06:03.7190307Z Traceback (most recent call last):</t>
         </is>
       </c>
       <c r="W32" s="19" t="inlineStr">
@@ -3794,12 +3732,12 @@
       </c>
       <c r="X32" s="19" t="inlineStr">
         <is>
-          <t>Set up job</t>
+          <t>Run GitHub Workflow Report</t>
         </is>
       </c>
       <c r="Y32" s="19" t="inlineStr">
         <is>
-          <t>Line 04</t>
+          <t>Line 06</t>
         </is>
       </c>
       <c r="Z32" s="19" t="inlineStr">
@@ -3831,12 +3769,12 @@
       </c>
       <c r="E33" s="19" t="inlineStr">
         <is>
-          <t>3046e3250b6d3bc90634487150d715e566686a47</t>
+          <t>372cfe624d49eb38f5e8baab2c748007dc54b018</t>
         </is>
       </c>
       <c r="F33" s="19" t="inlineStr">
         <is>
-          <t>Add demo.txt for testing purposes</t>
+          <t>Update demo.txt</t>
         </is>
       </c>
       <c r="G33" s="19" t="inlineStr">
@@ -3846,7 +3784,7 @@
       </c>
       <c r="H33" s="19" t="inlineStr">
         <is>
-          <t>2026-04-06T10:02:10Z</t>
+          <t>2026-04-06T10:04:34Z</t>
         </is>
       </c>
       <c r="I33" s="19" t="inlineStr">
@@ -3862,11 +3800,11 @@
       <c r="O33" s="19" t="inlineStr"/>
       <c r="P33" s="19" t="inlineStr">
         <is>
-          <t>.github/workflows/workflow_report.yml</t>
+          <t>GitHub Workflow Report</t>
         </is>
       </c>
       <c r="Q33" s="19" t="n">
-        <v>24027621196</v>
+        <v>24027694141</v>
       </c>
       <c r="R33" s="19" t="inlineStr">
         <is>
@@ -3875,7 +3813,7 @@
       </c>
       <c r="S33" s="19" t="inlineStr">
         <is>
-          <t>2026-04-06T10:02:12Z</t>
+          <t>2026-04-06T10:04:36Z</t>
         </is>
       </c>
       <c r="T33" s="19" t="inlineStr">
@@ -3890,14 +3828,22 @@
       </c>
       <c r="V33" s="19" t="inlineStr">
         <is>
-          <t>Failure (see logs)</t>
-        </is>
-      </c>
-      <c r="W33" s="19" t="inlineStr"/>
-      <c r="X33" s="19" t="inlineStr"/>
+          <t>Job 'report' step 'Set up job' failed — 2026-04-06T10:04:40.5244711Z ##[error]This request has been automatically failed because it uses a deprecated version of</t>
+        </is>
+      </c>
+      <c r="W33" s="19" t="inlineStr">
+        <is>
+          <t>report</t>
+        </is>
+      </c>
+      <c r="X33" s="19" t="inlineStr">
+        <is>
+          <t>Set up job</t>
+        </is>
+      </c>
       <c r="Y33" s="19" t="inlineStr">
         <is>
-          <t>See GitHub Actions logs</t>
+          <t>Line 04</t>
         </is>
       </c>
       <c r="Z33" s="19" t="inlineStr">
@@ -3929,12 +3875,12 @@
       </c>
       <c r="E34" s="19" t="inlineStr">
         <is>
-          <t>32de2be70035a86124e1345187c9ba078e4cf3bf</t>
+          <t>e7bf9d94f807df2e25e29ad5d30bc78e1b2fbd25</t>
         </is>
       </c>
       <c r="F34" s="19" t="inlineStr">
         <is>
-          <t>Add GitHub Workflow Report YAML configuration</t>
+          <t>Update workflow_report.yml</t>
         </is>
       </c>
       <c r="G34" s="19" t="inlineStr">
@@ -3944,7 +3890,7 @@
       </c>
       <c r="H34" s="19" t="inlineStr">
         <is>
-          <t>2026-04-06T10:01:02Z</t>
+          <t>2026-04-06T10:04:22Z</t>
         </is>
       </c>
       <c r="I34" s="19" t="inlineStr">
@@ -3960,180 +3906,384 @@
       <c r="O34" s="19" t="inlineStr"/>
       <c r="P34" s="19" t="inlineStr">
         <is>
+          <t>GitHub Workflow Report</t>
+        </is>
+      </c>
+      <c r="Q34" s="19" t="n">
+        <v>24027689526</v>
+      </c>
+      <c r="R34" s="19" t="inlineStr">
+        <is>
+          <t>push</t>
+        </is>
+      </c>
+      <c r="S34" s="19" t="inlineStr">
+        <is>
+          <t>2026-04-06T10:04:27Z</t>
+        </is>
+      </c>
+      <c r="T34" s="19" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="U34" s="20" t="inlineStr">
+        <is>
+          <t>failure</t>
+        </is>
+      </c>
+      <c r="V34" s="19" t="inlineStr">
+        <is>
+          <t>Job 'report' step 'Set up job' failed — 2026-04-06T10:04:31.3428173Z ##[error]This request has been automatically failed because it uses a deprecated version of</t>
+        </is>
+      </c>
+      <c r="W34" s="19" t="inlineStr">
+        <is>
+          <t>report</t>
+        </is>
+      </c>
+      <c r="X34" s="19" t="inlineStr">
+        <is>
+          <t>Set up job</t>
+        </is>
+      </c>
+      <c r="Y34" s="19" t="inlineStr">
+        <is>
+          <t>Line 04</t>
+        </is>
+      </c>
+      <c r="Z34" s="19" t="inlineStr">
+        <is>
+          <t>Review the full workflow log in GitHub Actions for the specific error message.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="19" t="inlineStr">
+        <is>
+          <t>git-report</t>
+        </is>
+      </c>
+      <c r="B35" s="19" t="inlineStr">
+        <is>
+          <t>vidyakar-whitedev</t>
+        </is>
+      </c>
+      <c r="C35" s="19" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="D35" s="19" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E35" s="19" t="inlineStr">
+        <is>
+          <t>3046e3250b6d3bc90634487150d715e566686a47</t>
+        </is>
+      </c>
+      <c r="F35" s="19" t="inlineStr">
+        <is>
+          <t>Add demo.txt for testing purposes</t>
+        </is>
+      </c>
+      <c r="G35" s="19" t="inlineStr">
+        <is>
+          <t>vidyakar-whitedev</t>
+        </is>
+      </c>
+      <c r="H35" s="19" t="inlineStr">
+        <is>
+          <t>2026-04-06T10:02:10Z</t>
+        </is>
+      </c>
+      <c r="I35" s="19" t="inlineStr">
+        <is>
+          <t>git-report-poc2</t>
+        </is>
+      </c>
+      <c r="J35" s="19" t="inlineStr"/>
+      <c r="K35" s="19" t="inlineStr"/>
+      <c r="L35" s="19" t="inlineStr"/>
+      <c r="M35" s="19" t="inlineStr"/>
+      <c r="N35" s="19" t="inlineStr"/>
+      <c r="O35" s="19" t="inlineStr"/>
+      <c r="P35" s="19" t="inlineStr">
+        <is>
           <t>.github/workflows/workflow_report.yml</t>
         </is>
       </c>
-      <c r="Q34" s="19" t="n">
+      <c r="Q35" s="19" t="n">
+        <v>24027621196</v>
+      </c>
+      <c r="R35" s="19" t="inlineStr">
+        <is>
+          <t>push</t>
+        </is>
+      </c>
+      <c r="S35" s="19" t="inlineStr">
+        <is>
+          <t>2026-04-06T10:02:12Z</t>
+        </is>
+      </c>
+      <c r="T35" s="19" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="U35" s="20" t="inlineStr">
+        <is>
+          <t>failure</t>
+        </is>
+      </c>
+      <c r="V35" s="19" t="inlineStr">
+        <is>
+          <t>Failure (see logs)</t>
+        </is>
+      </c>
+      <c r="W35" s="19" t="inlineStr"/>
+      <c r="X35" s="19" t="inlineStr"/>
+      <c r="Y35" s="19" t="inlineStr">
+        <is>
+          <t>See GitHub Actions logs</t>
+        </is>
+      </c>
+      <c r="Z35" s="19" t="inlineStr">
+        <is>
+          <t>Review the full workflow log in GitHub Actions for the specific error message.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="19" t="inlineStr">
+        <is>
+          <t>git-report</t>
+        </is>
+      </c>
+      <c r="B36" s="19" t="inlineStr">
+        <is>
+          <t>vidyakar-whitedev</t>
+        </is>
+      </c>
+      <c r="C36" s="19" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="D36" s="19" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E36" s="19" t="inlineStr">
+        <is>
+          <t>32de2be70035a86124e1345187c9ba078e4cf3bf</t>
+        </is>
+      </c>
+      <c r="F36" s="19" t="inlineStr">
+        <is>
+          <t>Add GitHub Workflow Report YAML configuration</t>
+        </is>
+      </c>
+      <c r="G36" s="19" t="inlineStr">
+        <is>
+          <t>vidyakar-whitedev</t>
+        </is>
+      </c>
+      <c r="H36" s="19" t="inlineStr">
+        <is>
+          <t>2026-04-06T10:01:02Z</t>
+        </is>
+      </c>
+      <c r="I36" s="19" t="inlineStr">
+        <is>
+          <t>git-report-poc2</t>
+        </is>
+      </c>
+      <c r="J36" s="19" t="inlineStr"/>
+      <c r="K36" s="19" t="inlineStr"/>
+      <c r="L36" s="19" t="inlineStr"/>
+      <c r="M36" s="19" t="inlineStr"/>
+      <c r="N36" s="19" t="inlineStr"/>
+      <c r="O36" s="19" t="inlineStr"/>
+      <c r="P36" s="19" t="inlineStr">
+        <is>
+          <t>.github/workflows/workflow_report.yml</t>
+        </is>
+      </c>
+      <c r="Q36" s="19" t="n">
         <v>24027587697</v>
       </c>
-      <c r="R34" s="19" t="inlineStr">
+      <c r="R36" s="19" t="inlineStr">
         <is>
           <t>push</t>
         </is>
       </c>
-      <c r="S34" s="19" t="inlineStr">
+      <c r="S36" s="19" t="inlineStr">
         <is>
           <t>2026-04-06T10:01:04Z</t>
         </is>
       </c>
-      <c r="T34" s="19" t="inlineStr">
+      <c r="T36" s="19" t="inlineStr">
         <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="U34" s="20" t="inlineStr">
+      <c r="U36" s="20" t="inlineStr">
         <is>
           <t>failure</t>
         </is>
       </c>
-      <c r="V34" s="19" t="inlineStr">
+      <c r="V36" s="19" t="inlineStr">
         <is>
           <t>Failure (see logs)</t>
         </is>
       </c>
-      <c r="W34" s="19" t="inlineStr"/>
-      <c r="X34" s="19" t="inlineStr"/>
-      <c r="Y34" s="19" t="inlineStr">
+      <c r="W36" s="19" t="inlineStr"/>
+      <c r="X36" s="19" t="inlineStr"/>
+      <c r="Y36" s="19" t="inlineStr">
         <is>
           <t>See GitHub Actions logs</t>
         </is>
       </c>
-      <c r="Z34" s="19" t="inlineStr">
+      <c r="Z36" s="19" t="inlineStr">
         <is>
           <t>Review the full workflow log in GitHub Actions for the specific error message.</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="18" t="inlineStr">
-        <is>
-          <t>git-report</t>
-        </is>
-      </c>
-      <c r="B35" s="18" t="inlineStr">
-        <is>
-          <t>vidyakar-whitedev</t>
-        </is>
-      </c>
-      <c r="C35" s="18" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="16" t="inlineStr">
+        <is>
+          <t>git-report</t>
+        </is>
+      </c>
+      <c r="B37" s="16" t="inlineStr">
+        <is>
+          <t>vidyakar-whitedev</t>
+        </is>
+      </c>
+      <c r="C37" s="16" t="inlineStr">
         <is>
           <t>public</t>
         </is>
       </c>
-      <c r="D35" s="18" t="inlineStr">
+      <c r="D37" s="16" t="inlineStr">
         <is>
           <t>main</t>
         </is>
       </c>
-      <c r="E35" s="18" t="inlineStr">
+      <c r="E37" s="16" t="inlineStr">
         <is>
           <t>8eaab42012c4f02192c65cf59561b5c261b2cf90</t>
         </is>
       </c>
-      <c r="F35" s="18" t="inlineStr">
+      <c r="F37" s="16" t="inlineStr">
         <is>
           <t>Create github_workflow_report.py</t>
         </is>
       </c>
-      <c r="G35" s="18" t="inlineStr">
-        <is>
-          <t>vidyakar-whitedev</t>
-        </is>
-      </c>
-      <c r="H35" s="18" t="inlineStr">
+      <c r="G37" s="16" t="inlineStr">
+        <is>
+          <t>vidyakar-whitedev</t>
+        </is>
+      </c>
+      <c r="H37" s="16" t="inlineStr">
         <is>
           <t>2026-04-06T09:50:41Z</t>
         </is>
       </c>
-      <c r="I35" s="18" t="inlineStr">
+      <c r="I37" s="16" t="inlineStr">
         <is>
           <t>git-report-poc2</t>
         </is>
       </c>
-      <c r="J35" s="18" t="inlineStr"/>
-      <c r="K35" s="18" t="inlineStr"/>
-      <c r="L35" s="18" t="inlineStr"/>
-      <c r="M35" s="18" t="inlineStr"/>
-      <c r="N35" s="18" t="inlineStr"/>
-      <c r="O35" s="18" t="inlineStr"/>
-      <c r="P35" s="18" t="inlineStr"/>
-      <c r="Q35" s="18" t="inlineStr"/>
-      <c r="R35" s="18" t="inlineStr"/>
-      <c r="S35" s="18" t="inlineStr"/>
-      <c r="T35" s="18" t="inlineStr"/>
-      <c r="U35" s="18" t="inlineStr"/>
-      <c r="V35" s="18" t="inlineStr"/>
-      <c r="W35" s="18" t="inlineStr"/>
-      <c r="X35" s="18" t="inlineStr"/>
-      <c r="Y35" s="18" t="inlineStr"/>
-      <c r="Z35" s="18" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="15" t="inlineStr">
-        <is>
-          <t>git-report</t>
-        </is>
-      </c>
-      <c r="B36" s="15" t="inlineStr">
-        <is>
-          <t>vidyakar-whitedev</t>
-        </is>
-      </c>
-      <c r="C36" s="15" t="inlineStr">
+      <c r="J37" s="16" t="inlineStr"/>
+      <c r="K37" s="16" t="inlineStr"/>
+      <c r="L37" s="16" t="inlineStr"/>
+      <c r="M37" s="16" t="inlineStr"/>
+      <c r="N37" s="16" t="inlineStr"/>
+      <c r="O37" s="16" t="inlineStr"/>
+      <c r="P37" s="16" t="inlineStr"/>
+      <c r="Q37" s="16" t="inlineStr"/>
+      <c r="R37" s="16" t="inlineStr"/>
+      <c r="S37" s="16" t="inlineStr"/>
+      <c r="T37" s="16" t="inlineStr"/>
+      <c r="U37" s="16" t="inlineStr"/>
+      <c r="V37" s="16" t="inlineStr"/>
+      <c r="W37" s="16" t="inlineStr"/>
+      <c r="X37" s="16" t="inlineStr"/>
+      <c r="Y37" s="16" t="inlineStr"/>
+      <c r="Z37" s="16" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="15" t="inlineStr">
+        <is>
+          <t>git-report</t>
+        </is>
+      </c>
+      <c r="B38" s="15" t="inlineStr">
+        <is>
+          <t>vidyakar-whitedev</t>
+        </is>
+      </c>
+      <c r="C38" s="15" t="inlineStr">
         <is>
           <t>public</t>
         </is>
       </c>
-      <c r="D36" s="15" t="inlineStr">
+      <c r="D38" s="15" t="inlineStr">
         <is>
           <t>main</t>
         </is>
       </c>
-      <c r="E36" s="15" t="inlineStr">
+      <c r="E38" s="15" t="inlineStr">
         <is>
           <t>a9e73f5e7cd8ea7da7f4969f80034915cc9f302c</t>
         </is>
       </c>
-      <c r="F36" s="15" t="inlineStr">
+      <c r="F38" s="15" t="inlineStr">
         <is>
           <t>Initial commit</t>
         </is>
       </c>
-      <c r="G36" s="15" t="inlineStr">
-        <is>
-          <t>vidyakar-whitedev</t>
-        </is>
-      </c>
-      <c r="H36" s="15" t="inlineStr">
+      <c r="G38" s="15" t="inlineStr">
+        <is>
+          <t>vidyakar-whitedev</t>
+        </is>
+      </c>
+      <c r="H38" s="15" t="inlineStr">
         <is>
           <t>2026-04-06T09:48:37Z</t>
         </is>
       </c>
-      <c r="I36" s="15" t="inlineStr">
+      <c r="I38" s="15" t="inlineStr">
         <is>
           <t>git-report-poc2</t>
         </is>
       </c>
-      <c r="J36" s="15" t="inlineStr"/>
-      <c r="K36" s="15" t="inlineStr"/>
-      <c r="L36" s="15" t="inlineStr"/>
-      <c r="M36" s="15" t="inlineStr"/>
-      <c r="N36" s="15" t="inlineStr"/>
-      <c r="O36" s="15" t="inlineStr"/>
-      <c r="P36" s="15" t="inlineStr"/>
-      <c r="Q36" s="15" t="inlineStr"/>
-      <c r="R36" s="15" t="inlineStr"/>
-      <c r="S36" s="15" t="inlineStr"/>
-      <c r="T36" s="15" t="inlineStr"/>
-      <c r="U36" s="15" t="inlineStr"/>
-      <c r="V36" s="15" t="inlineStr"/>
-      <c r="W36" s="15" t="inlineStr"/>
-      <c r="X36" s="15" t="inlineStr"/>
-      <c r="Y36" s="15" t="inlineStr"/>
-      <c r="Z36" s="15" t="inlineStr"/>
+      <c r="J38" s="15" t="inlineStr"/>
+      <c r="K38" s="15" t="inlineStr"/>
+      <c r="L38" s="15" t="inlineStr"/>
+      <c r="M38" s="15" t="inlineStr"/>
+      <c r="N38" s="15" t="inlineStr"/>
+      <c r="O38" s="15" t="inlineStr"/>
+      <c r="P38" s="15" t="inlineStr"/>
+      <c r="Q38" s="15" t="inlineStr"/>
+      <c r="R38" s="15" t="inlineStr"/>
+      <c r="S38" s="15" t="inlineStr"/>
+      <c r="T38" s="15" t="inlineStr"/>
+      <c r="U38" s="15" t="inlineStr"/>
+      <c r="V38" s="15" t="inlineStr"/>
+      <c r="W38" s="15" t="inlineStr"/>
+      <c r="X38" s="15" t="inlineStr"/>
+      <c r="Y38" s="15" t="inlineStr"/>
+      <c r="Z38" s="15" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Z36"/>
+  <autoFilter ref="A1:Z38"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5356,7 +5506,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="22" t="inlineStr">
         <is>
-          <t>Generated: 2026-04-10 16:37 UTC  |  GitHub Activity &amp; Workflow Audit Report</t>
+          <t>Generated: 2026-04-11 05:18 UTC  |  GitHub Activity &amp; Workflow Audit Report</t>
         </is>
       </c>
     </row>

</xml_diff>